<commit_message>
Restore complete architecture discovery methodology
</commit_message>
<xml_diff>
--- a/research/research_program.xlsx
+++ b/research/research_program.xlsx
@@ -2,15 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R89c7fd9716d14249"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phases" sheetId="2" r:id="Rce99aa118a45407d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiments" sheetId="3" r:id="Ree73747569a3457b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Knowledge" sheetId="4" r:id="R3f1737ec85e94dde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hypotheses" sheetId="5" r:id="R1d4df67ce26e4c1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="6" r:id="R39bdb2bc0f2f45d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architectures" sheetId="7" r:id="R12a171d28e5742e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicators" sheetId="8" r:id="Re2aa58404cbd45d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Literature" sheetId="9" r:id="R0492cdb881fb445e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R093c58795e6f4f4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phases" sheetId="2" r:id="R9b3d7f3a5d7f431a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiments" sheetId="3" r:id="R6a47c50318a8482d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Knowledge" sheetId="4" r:id="Rc1e0311440ca4992"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hypotheses" sheetId="5" r:id="R2fad708ce60142e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="6" r:id="R851d7f6dc39c4d28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architectures" sheetId="7" r:id="R1b0a8632adfd4172"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BiasTaxonomy" sheetId="8" r:id="R33c43f424c9d4c67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patterns" sheetId="9" r:id="R08967de534b24f3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="10" r:id="R83fc8c77ecdc4af7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evaluation" sheetId="11" r:id="R2f9e950f55f54e0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicators" sheetId="12" r:id="Rb2f8e263d92c45e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Literature" sheetId="13" r:id="R2d2c6fd1d4924dbb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -887,6 +891,2309 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="62" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="85" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
+      <x:c r="A1" s="17" t="str">
+        <x:v>Evidence-guided creative methodology</x:v>
+      </x:c>
+      <x:c r="B1" s="17"/>
+      <x:c r="C1" s="17"/>
+      <x:c r="D1" s="17"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="18"/>
+      <x:c r="B2" s="18"/>
+      <x:c r="C2" s="18"/>
+      <x:c r="D2" s="18"/>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="22" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B3" s="22" t="str">
+        <x:v>Type</x:v>
+      </x:c>
+      <x:c r="C3" s="22" t="str">
+        <x:v>Principle / Stage</x:v>
+      </x:c>
+      <x:c r="D3" s="22" t="str">
+        <x:v>Operational consequence / Output</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="23" t="str">
+        <x:v>M-A01</x:v>
+      </x:c>
+      <x:c r="B4" s="23" t="str">
+        <x:v>axiom</x:v>
+      </x:c>
+      <x:c r="C4" s="23" t="str">
+        <x:v>Existence is cheap; learnability is the real architectural property.</x:v>
+      </x:c>
+      <x:c r="D4" s="23" t="str">
+        <x:v>Universal approximation or representability cannot promote a model.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="23" t="str">
+        <x:v>M-A02</x:v>
+      </x:c>
+      <x:c r="B5" s="23" t="str">
+        <x:v>axiom</x:v>
+      </x:c>
+      <x:c r="C5" s="23" t="str">
+        <x:v>A benchmark score is a phenotype, not a mechanism.</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="str">
+        <x:v>Every promoted result needs deconvolution through diagnostics, probes or component tests.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="23" t="str">
+        <x:v>M-A03</x:v>
+      </x:c>
+      <x:c r="B6" s="23" t="str">
+        <x:v>axiom</x:v>
+      </x:c>
+      <x:c r="C6" s="23" t="str">
+        <x:v>Creativity is constrained recombination of established fragments.</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="str">
+        <x:v>Maintain a library of architectures, primitives and functional descriptors; generate multiple sketches.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="23" t="str">
+        <x:v>M-A04</x:v>
+      </x:c>
+      <x:c r="B7" s="23" t="str">
+        <x:v>axiom</x:v>
+      </x:c>
+      <x:c r="C7" s="23" t="str">
+        <x:v>Emergent component interactions are not fully predictable a priori.</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="str">
+        <x:v>Use empirical screening, then rationalize survivors instead of pretending first-principles certainty.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="23" t="str">
+        <x:v>M-A05</x:v>
+      </x:c>
+      <x:c r="B8" s="23" t="str">
+        <x:v>axiom</x:v>
+      </x:c>
+      <x:c r="C8" s="23" t="str">
+        <x:v>Mixed real tasks can hide capability differences below stochastic noise.</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="str">
+        <x:v>Use atomic synthetic playgrounds and mini-scaling laws before full-teacher claims.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="23" t="str">
+        <x:v>M-A06</x:v>
+      </x:c>
+      <x:c r="B9" s="23" t="str">
+        <x:v>axiom</x:v>
+      </x:c>
+      <x:c r="C9" s="23" t="str">
+        <x:v>Behavior and internal computation are separate objects of study.</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="str">
+        <x:v>Pair output metrics and qualitative plots with activation, gradient and causal probing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="23" t="str">
+        <x:v>M-A07</x:v>
+      </x:c>
+      <x:c r="B10" s="23" t="str">
+        <x:v>axiom</x:v>
+      </x:c>
+      <x:c r="C10" s="23" t="str">
+        <x:v>Information gained per experiment matters more than the number of runs.</x:v>
+      </x:c>
+      <x:c r="D10" s="23" t="str">
+        <x:v>Prefer orthogonal contrasts that eliminate branches of explanation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="23" t="str">
+        <x:v>M-A08</x:v>
+      </x:c>
+      <x:c r="B11" s="23" t="str">
+        <x:v>axiom</x:v>
+      </x:c>
+      <x:c r="C11" s="23" t="str">
+        <x:v>Synthetic discovery must resonate in the real target system.</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="str">
+        <x:v>Capability-bench hits require controlled full-teacher preflight and later scale/data confirmation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A12" s="23" t="str">
+        <x:v>MODE-RATIONAL</x:v>
+      </x:c>
+      <x:c r="B12" s="23" t="str">
+        <x:v>search mode</x:v>
+      </x:c>
+      <x:c r="C12" s="23" t="str">
+        <x:v>structure-based design: strong mathematical or biological prior exists</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="str">
+        <x:v>encode the prior in a standard architecture and test its causal benefit | Risk: correct static analogy but poor optimization dynamics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A13" s="23" t="str">
+        <x:v>MODE-ANALOGICAL</x:v>
+      </x:c>
+      <x:c r="B13" s="23" t="str">
+        <x:v>search mode</x:v>
+      </x:c>
+      <x:c r="C13" s="23" t="str">
+        <x:v>ligand-based design: successful architectures exist on related tasks</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="str">
+        <x:v>extract shared functional descriptors rather than copy whole models | Risk: cannot leave the neighborhood of known solutions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A14" s="23" t="str">
+        <x:v>MODE-PHENOTYPIC</x:v>
+      </x:c>
+      <x:c r="B14" s="23" t="str">
+        <x:v>search mode</x:v>
+      </x:c>
+      <x:c r="C14" s="23" t="str">
+        <x:v>phenotypic screening: mechanism is unknown</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="str">
+        <x:v>screen structurally diverse curated scaffolds on diagnostic phenotypes | Risk: benchmark chasing without target deconvolution</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A15" s="23" t="str">
+        <x:v>MODE-FRAGMENT</x:v>
+      </x:c>
+      <x:c r="B15" s="23" t="str">
+        <x:v>search mode</x:v>
+      </x:c>
+      <x:c r="C15" s="23" t="str">
+        <x:v>fragment-based design: candidate primitives can be isolated</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="str">
+        <x:v>test minimal fragments, then grow/link/merge only supported fragments | Risk: fragments that work alone may not compose</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A16" s="23" t="str">
+        <x:v>MODE-DENOVO</x:v>
+      </x:c>
+      <x:c r="B16" s="23" t="str">
+        <x:v>search mode</x:v>
+      </x:c>
+      <x:c r="C16" s="23" t="str">
+        <x:v>de-novo design: existing libraries cannot express a measured requirement</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="str">
+        <x:v>generate constrained compositions from established primitives | Risk: untrainable, uninterpretable or compute-inefficient inventions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="23" t="str">
+        <x:v>STAGE-01</x:v>
+      </x:c>
+      <x:c r="B17" s="23" t="str">
+        <x:v>creative stage</x:v>
+      </x:c>
+      <x:c r="C17" s="23" t="str">
+        <x:v>constraint_board</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="str">
+        <x:v>task contract, forbidden leakage, known dynamics, failure signatures, compute ceiling</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="23" t="str">
+        <x:v>STAGE-02</x:v>
+      </x:c>
+      <x:c r="B18" s="23" t="str">
+        <x:v>creative stage</x:v>
+      </x:c>
+      <x:c r="C18" s="23" t="str">
+        <x:v>atomic_decomposition</x:v>
+      </x:c>
+      <x:c r="D18" s="23" t="str">
+        <x:v>orthogonal capabilities and difficulty axes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="23" t="str">
+        <x:v>STAGE-03</x:v>
+      </x:c>
+      <x:c r="B19" s="23" t="str">
+        <x:v>creative stage</x:v>
+      </x:c>
+      <x:c r="C19" s="23" t="str">
+        <x:v>reference_retrieval</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="str">
+        <x:v>literature-grounded scaffold and primitive candidates from several taxonomy levels</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="23" t="str">
+        <x:v>STAGE-04</x:v>
+      </x:c>
+      <x:c r="B20" s="23" t="str">
+        <x:v>creative stage</x:v>
+      </x:c>
+      <x:c r="C20" s="23" t="str">
+        <x:v>sketch_generation</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="str">
+        <x:v>10-20 small candidate sketches covering diverse mechanisms, not cosmetic variants</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="23" t="str">
+        <x:v>STAGE-05</x:v>
+      </x:c>
+      <x:c r="B21" s="23" t="str">
+        <x:v>creative stage</x:v>
+      </x:c>
+      <x:c r="C21" s="23" t="str">
+        <x:v>cheap_screen</x:v>
+      </x:c>
+      <x:c r="D21" s="23" t="str">
+        <x:v>capability profiles on controlled microtasks; model-size x task-difficulty mini-scaling surfaces</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="23" t="str">
+        <x:v>STAGE-06</x:v>
+      </x:c>
+      <x:c r="B22" s="23" t="str">
+        <x:v>creative stage</x:v>
+      </x:c>
+      <x:c r="C22" s="23" t="str">
+        <x:v>hit_selection</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="str">
+        <x:v>2-3 survivors selected by multi-metric signatures and guardrails</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="23" t="str">
+        <x:v>STAGE-07</x:v>
+      </x:c>
+      <x:c r="B23" s="23" t="str">
+        <x:v>creative stage</x:v>
+      </x:c>
+      <x:c r="C23" s="23" t="str">
+        <x:v>target_deconvolution</x:v>
+      </x:c>
+      <x:c r="D23" s="23" t="str">
+        <x:v>probes, ablations and causal interventions explaining which mechanism is used</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="23" t="str">
+        <x:v>STAGE-08</x:v>
+      </x:c>
+      <x:c r="B24" s="23" t="str">
+        <x:v>creative stage</x:v>
+      </x:c>
+      <x:c r="C24" s="23" t="str">
+        <x:v>lead_optimization</x:v>
+      </x:c>
+      <x:c r="D24" s="23" t="str">
+        <x:v>one-factor rational refinements to a supported mechanism</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="A25" s="23" t="str">
+        <x:v>STAGE-09</x:v>
+      </x:c>
+      <x:c r="B25" s="23" t="str">
+        <x:v>creative stage</x:v>
+      </x:c>
+      <x:c r="C25" s="23" t="str">
+        <x:v>real_system_resonance</x:v>
+      </x:c>
+      <x:c r="D25" s="23" t="str">
+        <x:v>capacity-matched full-teacher validation across seeds and regimes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
+      <x:c r="A26" s="23" t="str">
+        <x:v>STAGE-10</x:v>
+      </x:c>
+      <x:c r="B26" s="23" t="str">
+        <x:v>creative stage</x:v>
+      </x:c>
+      <x:c r="C26" s="23" t="str">
+        <x:v>composition</x:v>
+      </x:c>
+      <x:c r="D26" s="23" t="str">
+        <x:v>only independently validated complementary components, plus monolithic control</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="15" hidden="0" customHeight="1">
+      <x:c r="A27" s="23" t="str">
+        <x:v>STAGE-11</x:v>
+      </x:c>
+      <x:c r="B27" s="23" t="str">
+        <x:v>creative stage</x:v>
+      </x:c>
+      <x:c r="C27" s="23" t="str">
+        <x:v>confirmation</x:v>
+      </x:c>
+      <x:c r="D27" s="23" t="str">
+        <x:v>data/compute scaling, OOD, rollout and one frozen test evaluation</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:D1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="32" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="85" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="55" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
+      <x:c r="A1" s="17" t="str">
+        <x:v>Granular evaluation and observation taxonomy</x:v>
+      </x:c>
+      <x:c r="B1" s="17"/>
+      <x:c r="C1" s="17"/>
+      <x:c r="D1" s="17"/>
+      <x:c r="E1" s="17"/>
+      <x:c r="F1" s="17"/>
+      <x:c r="G1" s="17"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="18"/>
+      <x:c r="B2" s="18"/>
+      <x:c r="C2" s="18"/>
+      <x:c r="D2" s="18"/>
+      <x:c r="E2" s="18"/>
+      <x:c r="F2" s="18"/>
+      <x:c r="G2" s="18"/>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="22" t="str">
+        <x:v>Layer ID</x:v>
+      </x:c>
+      <x:c r="B3" s="22" t="str">
+        <x:v>Evaluation layer</x:v>
+      </x:c>
+      <x:c r="C3" s="22" t="str">
+        <x:v>Dimension ID</x:v>
+      </x:c>
+      <x:c r="D3" s="22" t="str">
+        <x:v>Dimension</x:v>
+      </x:c>
+      <x:c r="E3" s="22" t="str">
+        <x:v>Measures</x:v>
+      </x:c>
+      <x:c r="F3" s="22" t="str">
+        <x:v>Stratification axes</x:v>
+      </x:c>
+      <x:c r="G3" s="22" t="str">
+        <x:v>Warning</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="23" t="str">
+        <x:v>EV-BEHAVIOR</x:v>
+      </x:c>
+      <x:c r="B4" s="23" t="str">
+        <x:v>external behavior</x:v>
+      </x:c>
+      <x:c r="C4" s="23" t="str">
+        <x:v>EV-POINT</x:v>
+      </x:c>
+      <x:c r="D4" s="23" t="str">
+        <x:v>pointwise state fidelity</x:v>
+      </x:c>
+      <x:c r="E4" s="23" t="str">
+        <x:v>MAE; RMSE; normalized RMSE; bias; correlation; worst-coordinate error</x:v>
+      </x:c>
+      <x:c r="F4" s="23" t="str">
+        <x:v>state; state family; compartment; regime; trajectory; time since event</x:v>
+      </x:c>
+      <x:c r="G4" s="23" t="str"/>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="23" t="str">
+        <x:v>EV-BEHAVIOR</x:v>
+      </x:c>
+      <x:c r="B5" s="23" t="str">
+        <x:v>external behavior</x:v>
+      </x:c>
+      <x:c r="C5" s="23" t="str">
+        <x:v>EV-DIST</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="str">
+        <x:v>residual distribution</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="str">
+        <x:v>quantiles; skewness; kurtosis; tail index; heteroscedasticity; conditional bias; error autocorrelation</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="str">
+        <x:v>state family; regime; amplitude bin; input density</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="str"/>
+    </x:row>
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A6" s="23" t="str">
+        <x:v>EV-BEHAVIOR</x:v>
+      </x:c>
+      <x:c r="B6" s="23" t="str">
+        <x:v>external behavior</x:v>
+      </x:c>
+      <x:c r="C6" s="23" t="str">
+        <x:v>EV-EVENT</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="str">
+        <x:v>event morphology</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="str">
+        <x:v>precision; recall; F1; count error; peak amplitude error; peak-time error; rise/decay slope error; width; area; after-hyperpolarization; burst inter-spike interval; rapid-fire continuation/miss</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="str">
+        <x:v>isolated spike; burst; rapid fire; plateau-associated; compartment</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="str"/>
+    </x:row>
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A7" s="23" t="str">
+        <x:v>EV-BEHAVIOR</x:v>
+      </x:c>
+      <x:c r="B7" s="23" t="str">
+        <x:v>external behavior</x:v>
+      </x:c>
+      <x:c r="C7" s="23" t="str">
+        <x:v>EV-FREQ</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="str">
+        <x:v>frequency and multiresolution</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="str">
+        <x:v>band power ratio; PSD distance; spectral coherence; cross-spectrum; STFT distance; wavelet energy by scale; phase lag</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="str">
+        <x:v>state; regime; frequency band; event window</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="str"/>
+    </x:row>
+    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A8" s="23" t="str">
+        <x:v>EV-BEHAVIOR</x:v>
+      </x:c>
+      <x:c r="B8" s="23" t="str">
+        <x:v>external behavior</x:v>
+      </x:c>
+      <x:c r="C8" s="23" t="str">
+        <x:v>EV-ROLL</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="str">
+        <x:v>closed-loop rollout</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="str">
+        <x:v>horizon RMSE curve; error AUC; first divergence time; event survival by horizon; boundedness; state-family drift rate; error growth exponent</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="str">
+        <x:v>initial regime; input continuation; state family; horizon</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="str"/>
+    </x:row>
+    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A9" s="23" t="str">
+        <x:v>EV-BEHAVIOR</x:v>
+      </x:c>
+      <x:c r="B9" s="23" t="str">
+        <x:v>external behavior</x:v>
+      </x:c>
+      <x:c r="C9" s="23" t="str">
+        <x:v>EV-DYN</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="str">
+        <x:v>dynamical geometry</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="str">
+        <x:v>phase portrait discrepancy; delay-embedding geometry; recurrence rate; determinism; laminarity; trapping time; Lyapunov-style local divergence estimate; attractor occupancy; transition matrix</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="str">
+        <x:v>regime; embedding parameters; trajectory</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="str"/>
+    </x:row>
+    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A10" s="23" t="str">
+        <x:v>EV-BEHAVIOR</x:v>
+      </x:c>
+      <x:c r="B10" s="23" t="str">
+        <x:v>external behavior</x:v>
+      </x:c>
+      <x:c r="C10" s="23" t="str">
+        <x:v>EV-SPATIAL</x:v>
+      </x:c>
+      <x:c r="D10" s="23" t="str">
+        <x:v>four-compartment propagation</x:v>
+      </x:c>
+      <x:c r="E10" s="23" t="str">
+        <x:v>lag-conditioned transfer error; cross-compartment coherence; attenuation/amplification error; directionality; local versus propagated event error</x:v>
+      </x:c>
+      <x:c r="F10" s="23" t="str">
+        <x:v>source compartment; target compartment; path distance; input region</x:v>
+      </x:c>
+      <x:c r="G10" s="23" t="str"/>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="23" t="str">
+        <x:v>EV-BEHAVIOR</x:v>
+      </x:c>
+      <x:c r="B11" s="23" t="str">
+        <x:v>external behavior</x:v>
+      </x:c>
+      <x:c r="C11" s="23" t="str">
+        <x:v>EV-PROB</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="str">
+        <x:v>uncertainty and calibration</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="str">
+        <x:v>predictive interval coverage; negative log likelihood; calibration error; sharpness; coverage by regime</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="str">
+        <x:v>regime; state family; horizon</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="str"/>
+    </x:row>
+    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A12" s="23" t="str">
+        <x:v>EV-BEHAVIOR</x:v>
+      </x:c>
+      <x:c r="B12" s="23" t="str">
+        <x:v>external behavior</x:v>
+      </x:c>
+      <x:c r="C12" s="23" t="str">
+        <x:v>EV-ROBUST</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="str">
+        <x:v>robustness and generalization</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="str">
+        <x:v>OOD regime error; input-rate shift; timing jitter sensitivity; missing-channel sensitivity; initial-state perturbation; parameter-noise sensitivity</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="str">
+        <x:v>shift type; severity; state family</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="str"/>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="23" t="str">
+        <x:v>EV-BEHAVIOR</x:v>
+      </x:c>
+      <x:c r="B13" s="23" t="str">
+        <x:v>external behavior</x:v>
+      </x:c>
+      <x:c r="C13" s="23" t="str">
+        <x:v>EV-EFF</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="str">
+        <x:v>efficiency</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="str">
+        <x:v>parameters; FLOPs; wall time; peak memory; examples to threshold; updates to threshold; energy when available</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="str">
+        <x:v>model size; data fraction; difficulty</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="str"/>
+    </x:row>
+    <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A14" s="23" t="str">
+        <x:v>EV-INTERNAL</x:v>
+      </x:c>
+      <x:c r="B14" s="23" t="str">
+        <x:v>single-network internal computation</x:v>
+      </x:c>
+      <x:c r="C14" s="23" t="str">
+        <x:v>INT-ACT</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="str">
+        <x:v>activation distributions</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="str">
+        <x:v>mean; standard deviation; quantiles; skewness; kurtosis; entropy; sparsity; dead fraction; saturated fraction; derivative magnitude</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="str">
+        <x:v>layer; channel; time; regime; state family</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="str"/>
+    </x:row>
+    <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A15" s="23" t="str">
+        <x:v>EV-INTERNAL</x:v>
+      </x:c>
+      <x:c r="B15" s="23" t="str">
+        <x:v>single-network internal computation</x:v>
+      </x:c>
+      <x:c r="C15" s="23" t="str">
+        <x:v>INT-GATE</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="str">
+        <x:v>gates and memory</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="str">
+        <x:v>gate mean/entropy; open/closed fraction; time constant proxy; memory autocorrelation; reset/update coupling; event-conditioned trajectories</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="str">
+        <x:v>cell; layer; regime; time to event</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="str"/>
+    </x:row>
+    <x:row r="16" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A16" s="23" t="str">
+        <x:v>EV-INTERNAL</x:v>
+      </x:c>
+      <x:c r="B16" s="23" t="str">
+        <x:v>single-network internal computation</x:v>
+      </x:c>
+      <x:c r="C16" s="23" t="str">
+        <x:v>INT-GEOM</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="str">
+        <x:v>representation geometry</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="str">
+        <x:v>effective rank; participation ratio; singular spectrum; CKA/RSA; class/regime separation; trajectory curvature; latent recurrence</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="str">
+        <x:v>layer; regime; training time</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="str"/>
+    </x:row>
+    <x:row r="17" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A17" s="23" t="str">
+        <x:v>EV-INTERNAL</x:v>
+      </x:c>
+      <x:c r="B17" s="23" t="str">
+        <x:v>single-network internal computation</x:v>
+      </x:c>
+      <x:c r="C17" s="23" t="str">
+        <x:v>INT-PROBE</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="str">
+        <x:v>decodability probes</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="str">
+        <x:v>linear probe; nonlinear probe control; phase decoding; state-family decoding; future-event decoding; compartment-source decoding</x:v>
+      </x:c>
+      <x:c r="F17" s="23" t="str">
+        <x:v>layer; lag; probe capacity</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="str">
+        <x:v>decodability is evidence of presence, not causal use</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A18" s="23" t="str">
+        <x:v>EV-INTERNAL</x:v>
+      </x:c>
+      <x:c r="B18" s="23" t="str">
+        <x:v>single-network internal computation</x:v>
+      </x:c>
+      <x:c r="C18" s="23" t="str">
+        <x:v>INT-CAUSAL</x:v>
+      </x:c>
+      <x:c r="D18" s="23" t="str">
+        <x:v>causal representation use</x:v>
+      </x:c>
+      <x:c r="E18" s="23" t="str">
+        <x:v>activation patching; channel ablation; state clamping; counterfactual intervention; mediated effect</x:v>
+      </x:c>
+      <x:c r="F18" s="23" t="str">
+        <x:v>layer; time; regime</x:v>
+      </x:c>
+      <x:c r="G18" s="23" t="str">
+        <x:v>interventions must remain inside the causal information contract</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A19" s="23" t="str">
+        <x:v>EV-INTERNAL</x:v>
+      </x:c>
+      <x:c r="B19" s="23" t="str">
+        <x:v>single-network internal computation</x:v>
+      </x:c>
+      <x:c r="C19" s="23" t="str">
+        <x:v>INT-JAC</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="str">
+        <x:v>local dynamics and sensitivity</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="str">
+        <x:v>input Jacobian spectrum; hidden-state Jacobian spectrum; spectral radius; singular values; local Lipschitz proxy; gradient propagation by lag</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="str">
+        <x:v>regime; state; layer; time</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="str"/>
+    </x:row>
+    <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A20" s="23" t="str">
+        <x:v>EV-TRAIN</x:v>
+      </x:c>
+      <x:c r="B20" s="23" t="str">
+        <x:v>training and optimization</x:v>
+      </x:c>
+      <x:c r="C20" s="23" t="str">
+        <x:v>TR-CURVE</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="str">
+        <x:v>learning curves</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="str">
+        <x:v>train/validation loss by update; component losses; regime metrics by update; time-to-threshold; overfit gap; grokking/delayed emergence</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="str">
+        <x:v>seed; learning rate; difficulty; model size</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="str"/>
+    </x:row>
+    <x:row r="21" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A21" s="23" t="str">
+        <x:v>EV-TRAIN</x:v>
+      </x:c>
+      <x:c r="B21" s="23" t="str">
+        <x:v>training and optimization</x:v>
+      </x:c>
+      <x:c r="C21" s="23" t="str">
+        <x:v>TR-GRAD</x:v>
+      </x:c>
+      <x:c r="D21" s="23" t="str">
+        <x:v>gradient and update flow</x:v>
+      </x:c>
+      <x:c r="E21" s="23" t="str">
+        <x:v>gradient norm; variance; signal-to-noise; update-to-weight ratio; clipping fraction; per-block norm; cross-objective cosine; Fisher diagonal proxy</x:v>
+      </x:c>
+      <x:c r="F21" s="23" t="str">
+        <x:v>parameter block; regime; loss component; training phase</x:v>
+      </x:c>
+      <x:c r="G21" s="23" t="str"/>
+    </x:row>
+    <x:row r="22" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A22" s="23" t="str">
+        <x:v>EV-TRAIN</x:v>
+      </x:c>
+      <x:c r="B22" s="23" t="str">
+        <x:v>training and optimization</x:v>
+      </x:c>
+      <x:c r="C22" s="23" t="str">
+        <x:v>TR-LAND</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="str">
+        <x:v>loss landscape</x:v>
+      </x:c>
+      <x:c r="E22" s="23" t="str">
+        <x:v>filter-normalized slices; initial-final interpolation; sharpness; Hessian top eigenvalue; Hessian trace; anisotropy; mode connectivity; noise sensitivity</x:v>
+      </x:c>
+      <x:c r="F22" s="23" t="str">
+        <x:v>regime loss; checkpoint; seed</x:v>
+      </x:c>
+      <x:c r="G22" s="23" t="str"/>
+    </x:row>
+    <x:row r="23" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A23" s="23" t="str">
+        <x:v>EV-TRAIN</x:v>
+      </x:c>
+      <x:c r="B23" s="23" t="str">
+        <x:v>training and optimization</x:v>
+      </x:c>
+      <x:c r="C23" s="23" t="str">
+        <x:v>TR-STOCH</x:v>
+      </x:c>
+      <x:c r="D23" s="23" t="str">
+        <x:v>stochastic stability</x:v>
+      </x:c>
+      <x:c r="E23" s="23" t="str">
+        <x:v>between-seed variance; nearby-learning-rate variance; data-order variance; bootstrap confidence intervals; rank stability; effect-size distribution</x:v>
+      </x:c>
+      <x:c r="F23" s="23" t="str">
+        <x:v>metric; difficulty; capacity</x:v>
+      </x:c>
+      <x:c r="G23" s="23" t="str"/>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="23" t="str">
+        <x:v>EV-CAPABILITY</x:v>
+      </x:c>
+      <x:c r="B24" s="23" t="str">
+        <x:v>capability profiles and mini-scaling laws</x:v>
+      </x:c>
+      <x:c r="C24" s="23" t="str">
+        <x:v>CAP-SURFACE</x:v>
+      </x:c>
+      <x:c r="D24" s="23" t="str">
+        <x:v>capacity x difficulty surface</x:v>
+      </x:c>
+      <x:c r="E24" s="23" t="str">
+        <x:v>success surface; transition boundary; slope with capacity; slope with difficulty; seed uncertainty</x:v>
+      </x:c>
+      <x:c r="F24" s="23" t="str"/>
+      <x:c r="G24" s="23" t="str"/>
+    </x:row>
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="A25" s="23" t="str">
+        <x:v>EV-CAPABILITY</x:v>
+      </x:c>
+      <x:c r="B25" s="23" t="str">
+        <x:v>capability profiles and mini-scaling laws</x:v>
+      </x:c>
+      <x:c r="C25" s="23" t="str">
+        <x:v>CAP-DATA</x:v>
+      </x:c>
+      <x:c r="D25" s="23" t="str">
+        <x:v>data efficiency surface</x:v>
+      </x:c>
+      <x:c r="E25" s="23" t="str">
+        <x:v>metric versus examples; metric versus event count; area under learning curve; minimum data to guardrail</x:v>
+      </x:c>
+      <x:c r="F25" s="23" t="str"/>
+      <x:c r="G25" s="23" t="str"/>
+    </x:row>
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
+      <x:c r="A26" s="23" t="str">
+        <x:v>EV-CAPABILITY</x:v>
+      </x:c>
+      <x:c r="B26" s="23" t="str">
+        <x:v>capability profiles and mini-scaling laws</x:v>
+      </x:c>
+      <x:c r="C26" s="23" t="str">
+        <x:v>CAP-COMP</x:v>
+      </x:c>
+      <x:c r="D26" s="23" t="str">
+        <x:v>compositional generalization</x:v>
+      </x:c>
+      <x:c r="E26" s="23" t="str">
+        <x:v>held-out mechanism combinations; length/horizon extrapolation; unseen event-density combinations</x:v>
+      </x:c>
+      <x:c r="F26" s="23" t="str"/>
+      <x:c r="G26" s="23" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="8" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="40" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="42" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="46" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
+      <x:c r="A1" s="17" t="str">
+        <x:v>Diagnostic and intervention catalog</x:v>
+      </x:c>
+      <x:c r="B1" s="17"/>
+      <x:c r="C1" s="17"/>
+      <x:c r="D1" s="17"/>
+      <x:c r="E1" s="17"/>
+      <x:c r="F1" s="17"/>
+      <x:c r="G1" s="17"/>
+      <x:c r="H1" s="17"/>
+      <x:c r="I1" s="17"/>
+      <x:c r="J1" s="17"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="18"/>
+      <x:c r="B2" s="18"/>
+      <x:c r="C2" s="18"/>
+      <x:c r="D2" s="18"/>
+      <x:c r="E2" s="18"/>
+      <x:c r="F2" s="18"/>
+      <x:c r="G2" s="18"/>
+      <x:c r="H2" s="18"/>
+      <x:c r="I2" s="18"/>
+      <x:c r="J2" s="18"/>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="22" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B3" s="22" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="C3" s="22" t="str">
+        <x:v>Tier</x:v>
+      </x:c>
+      <x:c r="D3" s="22" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="E3" s="22" t="str">
+        <x:v>Question</x:v>
+      </x:c>
+      <x:c r="F3" s="22" t="str">
+        <x:v>Method</x:v>
+      </x:c>
+      <x:c r="G3" s="22" t="str">
+        <x:v>Controls</x:v>
+      </x:c>
+      <x:c r="H3" s="22" t="str">
+        <x:v>Trigger</x:v>
+      </x:c>
+      <x:c r="I3" s="22" t="str">
+        <x:v>Authorized interventions</x:v>
+      </x:c>
+      <x:c r="J3" s="22" t="str">
+        <x:v>Interpretation limits</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A4" s="23" t="str">
+        <x:v>OUT-EVENT</x:v>
+      </x:c>
+      <x:c r="B4" s="23" t="str">
+        <x:v>output</x:v>
+      </x:c>
+      <x:c r="C4" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D4" s="23" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="E4" s="23" t="str">
+        <x:v>Are rare transitions recovered in amplitude, timing and count?</x:v>
+      </x:c>
+      <x:c r="F4" s="23" t="str">
+        <x:v>precision/recall/F1, peak error, event-window RMSE and phase error</x:v>
+      </x:c>
+      <x:c r="G4" s="23" t="str">
+        <x:v>fixed threshold | tolerance sweep | teacher event count</x:v>
+      </x:c>
+      <x:c r="H4" s="23" t="str">
+        <x:v>zero recall or amplitude compression</x:v>
+      </x:c>
+      <x:c r="I4" s="23" t="str">
+        <x:v>DG-01; TR-01; LO-02; SR-01</x:v>
+      </x:c>
+      <x:c r="J4" s="23" t="str">
+        <x:v>threshold metrics alone do not measure subthreshold fidelity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A5" s="23" t="str">
+        <x:v>OUT-ROLL</x:v>
+      </x:c>
+      <x:c r="B5" s="23" t="str">
+        <x:v>output</x:v>
+      </x:c>
+      <x:c r="C5" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="str">
+        <x:v>How does error grow under closed-loop rollout?</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="str">
+        <x:v>horizon-conditioned NRMSE and first-threshold-crossing divergence</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="str">
+        <x:v>same initial context | no teacher forcing after initialization</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="str">
+        <x:v>superlinear drift or family-specific divergence</x:v>
+      </x:c>
+      <x:c r="I5" s="23" t="str">
+        <x:v>SR-01; LO-03</x:v>
+      </x:c>
+      <x:c r="J5" s="23" t="str">
+        <x:v>finite horizons are task definitions, not universal stability proofs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A6" s="23" t="str">
+        <x:v>LL-INTERP</x:v>
+      </x:c>
+      <x:c r="B6" s="23" t="str">
+        <x:v>loss_landscape</x:v>
+      </x:c>
+      <x:c r="C6" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="str">
+        <x:v>preregistered</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="str">
+        <x:v>Does training cross a barrier into a smooth low-frequency basin?</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="str">
+        <x:v>loss along filter-normalized initial-to-final and paired-checkpoint interpolation</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="str">
+        <x:v>frozen validation batches by regime | BatchNorm statistics frozen | no test data</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="str">
+        <x:v>event loss barrier absent from common-regime loss</x:v>
+      </x:c>
+      <x:c r="I6" s="23" t="str">
+        <x:v>OP-01; LO-02</x:v>
+      </x:c>
+      <x:c r="J6" s="23" t="str">
+        <x:v>a 1-D path is not the full landscape</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A7" s="23" t="str">
+        <x:v>LL-SLICE</x:v>
+      </x:c>
+      <x:c r="B7" s="23" t="str">
+        <x:v>loss_landscape</x:v>
+      </x:c>
+      <x:c r="C7" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="str">
+        <x:v>preregistered</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="str">
+        <x:v>Are local neighborhoods sharp, anisotropic or regime-dependent?</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="str">
+        <x:v>filter-normalized 1-D/2-D random-direction slices</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="str">
+        <x:v>same perturbation radii | multiple direction seeds | parameter-group report</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="str">
+        <x:v>event curvature differs strongly from global curvature</x:v>
+      </x:c>
+      <x:c r="I7" s="23" t="str">
+        <x:v>RG-01; OP-01</x:v>
+      </x:c>
+      <x:c r="J7" s="23" t="str">
+        <x:v>visual roughness depends on direction sampling</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A8" s="23" t="str">
+        <x:v>LL-HESS-TOP</x:v>
+      </x:c>
+      <x:c r="B8" s="23" t="str">
+        <x:v>loss_landscape</x:v>
+      </x:c>
+      <x:c r="C8" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="str">
+        <x:v>preregistered</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="str">
+        <x:v>What is the strongest local curvature?</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="str">
+        <x:v>Hessian-vector products with power iteration/Lanczos</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="str">
+        <x:v>same frozen batches | convergence residual | parameter normalization</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="str">
+        <x:v>large event-conditioned eigenvalue or scaffold-specific curvature spike</x:v>
+      </x:c>
+      <x:c r="I8" s="23" t="str">
+        <x:v>OP-01; RG-01</x:v>
+      </x:c>
+      <x:c r="J8" s="23" t="str">
+        <x:v>largest eigenvalue omits most directions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="23" t="str">
+        <x:v>LL-HESS-TRACE</x:v>
+      </x:c>
+      <x:c r="B9" s="23" t="str">
+        <x:v>loss_landscape</x:v>
+      </x:c>
+      <x:c r="C9" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="str">
+        <x:v>preregistered</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="str">
+        <x:v>How much aggregate curvature is present?</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="str">
+        <x:v>Hutchinson trace estimate with confidence interval</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="str">
+        <x:v>fixed probe seeds | probe-count convergence</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="str">
+        <x:v>large trace with high anisotropy</x:v>
+      </x:c>
+      <x:c r="I9" s="23" t="str">
+        <x:v>OP-01; RG-01</x:v>
+      </x:c>
+      <x:c r="J9" s="23" t="str">
+        <x:v>stochastic estimator and parameterization dependent</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A10" s="23" t="str">
+        <x:v>GR-CONFLICT</x:v>
+      </x:c>
+      <x:c r="B10" s="23" t="str">
+        <x:v>gradient</x:v>
+      </x:c>
+      <x:c r="C10" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D10" s="23" t="str">
+        <x:v>preregistered</x:v>
+      </x:c>
+      <x:c r="E10" s="23" t="str">
+        <x:v>Do event, subthreshold, slow and synaptic objectives request opposing updates?</x:v>
+      </x:c>
+      <x:c r="F10" s="23" t="str">
+        <x:v>pairwise gradient cosine matrix by parameter block</x:v>
+      </x:c>
+      <x:c r="G10" s="23" t="str">
+        <x:v>identical examples | loss-scale normalized companion view | bootstrap intervals</x:v>
+      </x:c>
+      <x:c r="H10" s="23" t="str">
+        <x:v>stable negative cosine or extreme norm imbalance</x:v>
+      </x:c>
+      <x:c r="I10" s="23" t="str">
+        <x:v>LO-02; LO-04; TR-01</x:v>
+      </x:c>
+      <x:c r="J10" s="23" t="str">
+        <x:v>local conflicts do not prove global incompatibility</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A11" s="23" t="str">
+        <x:v>GR-SNR</x:v>
+      </x:c>
+      <x:c r="B11" s="23" t="str">
+        <x:v>gradient</x:v>
+      </x:c>
+      <x:c r="C11" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="str">
+        <x:v>preregistered</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="str">
+        <x:v>Is the rare-event gradient visible above minibatch noise?</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="str">
+        <x:v>per-regime gradient norm, variance and signal-to-noise ratio</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="str">
+        <x:v>equal example counts | multiple minibatches</x:v>
+      </x:c>
+      <x:c r="H11" s="23" t="str">
+        <x:v>event gradient SNR low or contribution negligible</x:v>
+      </x:c>
+      <x:c r="I11" s="23" t="str">
+        <x:v>TR-01; LO-02</x:v>
+      </x:c>
+      <x:c r="J11" s="23" t="str">
+        <x:v>estimator depends on batching</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A12" s="23" t="str">
+        <x:v>ACT-SEP</x:v>
+      </x:c>
+      <x:c r="B12" s="23" t="str">
+        <x:v>activation</x:v>
+      </x:c>
+      <x:c r="C12" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="str">
+        <x:v>planned</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="str">
+        <x:v>Where does event/non-event separability appear and disappear?</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="str">
+        <x:v>linear probes and distribution distances per layer/time lag</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="str">
+        <x:v>held-out validation trajectories | probe capacity fixed</x:v>
+      </x:c>
+      <x:c r="H12" s="23" t="str">
+        <x:v>early separability followed by readout collapse</x:v>
+      </x:c>
+      <x:c r="I12" s="23" t="str">
+        <x:v>SR-01; HY-01</x:v>
+      </x:c>
+      <x:c r="J12" s="23" t="str">
+        <x:v>decodability is not causal use</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="23" t="str">
+        <x:v>ACT-SAT</x:v>
+      </x:c>
+      <x:c r="B13" s="23" t="str">
+        <x:v>activation</x:v>
+      </x:c>
+      <x:c r="C13" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="str">
+        <x:v>planned</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="str">
+        <x:v>Do nonlinearities or gates saturate in the failed regime?</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="str">
+        <x:v>quantiles, dead/saturated fraction, gate entropy and derivatives</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="str">
+        <x:v>regime conditioning | same checkpoints</x:v>
+      </x:c>
+      <x:c r="H13" s="23" t="str">
+        <x:v>event-specific saturation with gradient attenuation</x:v>
+      </x:c>
+      <x:c r="I13" s="23" t="str">
+        <x:v>AC-01; NM-01</x:v>
+      </x:c>
+      <x:c r="J13" s="23" t="str">
+        <x:v>saturation may be adaptive rather than pathological</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A14" s="23" t="str">
+        <x:v>ACT-RANK</x:v>
+      </x:c>
+      <x:c r="B14" s="23" t="str">
+        <x:v>activation</x:v>
+      </x:c>
+      <x:c r="C14" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="str">
+        <x:v>planned</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="str">
+        <x:v>Does the latent collapse to a low-dimensional smooth manifold?</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="str">
+        <x:v>effective rank, participation ratio and singular spectrum by regime</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="str">
+        <x:v>center/scale conventions | matched sample count</x:v>
+      </x:c>
+      <x:c r="H14" s="23" t="str">
+        <x:v>event trajectories require directions absent in prediction latent</x:v>
+      </x:c>
+      <x:c r="I14" s="23" t="str">
+        <x:v>SC-05; SR-01</x:v>
+      </x:c>
+      <x:c r="J14" s="23" t="str">
+        <x:v>rank depends on coordinate scaling</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A15" s="23" t="str">
+        <x:v>DYN-RQA</x:v>
+      </x:c>
+      <x:c r="B15" s="23" t="str">
+        <x:v>dynamics</x:v>
+      </x:c>
+      <x:c r="C15" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="str">
+        <x:v>Does the surrogate preserve recurrent dynamical structure?</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="str">
+        <x:v>recurrence plots, recurrence rate, determinism and laminarity</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="str">
+        <x:v>shared embedding rule | threshold sensitivity</x:v>
+      </x:c>
+      <x:c r="H15" s="23" t="str">
+        <x:v>regime-specific topology mismatch</x:v>
+      </x:c>
+      <x:c r="I15" s="23" t="str">
+        <x:v>SC-05; SC-06</x:v>
+      </x:c>
+      <x:c r="J15" s="23" t="str">
+        <x:v>Takens-style reconstruction assumptions must be stated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A16" s="23" t="str">
+        <x:v>LL-MODE</x:v>
+      </x:c>
+      <x:c r="B16" s="23" t="str">
+        <x:v>loss_landscape</x:v>
+      </x:c>
+      <x:c r="C16" s="23" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="str">
+        <x:v>conditional</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="str">
+        <x:v>Are independently trained solutions connected by low-loss paths?</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="str">
+        <x:v>linear and polygonal mode connectivity</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="str">
+        <x:v>permutation alignment | same data and objective</x:v>
+      </x:c>
+      <x:c r="H16" s="23" t="str">
+        <x:v>seed instability plus distinct basins in Tier 1</x:v>
+      </x:c>
+      <x:c r="I16" s="23" t="str">
+        <x:v>OP-01</x:v>
+      </x:c>
+      <x:c r="J16" s="23" t="str">
+        <x:v>connectivity can change under symmetry alignment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A17" s="23" t="str">
+        <x:v>LL-FRACTAL</x:v>
+      </x:c>
+      <x:c r="B17" s="23" t="str">
+        <x:v>loss_landscape</x:v>
+      </x:c>
+      <x:c r="C17" s="23" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="str">
+        <x:v>conditional</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="str">
+        <x:v>Is apparent roughness scale-dependent?</x:v>
+      </x:c>
+      <x:c r="F17" s="23" t="str">
+        <x:v>wavelet spectrum, Hölder/fractal or multifractal estimators on controlled slices</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="str">
+        <x:v>large scale range | synthetic calibration surfaces | uncertainty</x:v>
+      </x:c>
+      <x:c r="H17" s="23" t="str">
+        <x:v>unresolved multi-scale roughness after Tier 1</x:v>
+      </x:c>
+      <x:c r="I17" s="23" t="str"/>
+      <x:c r="J17" s="23" t="str">
+        <x:v>high estimator variance and weak direct intervention mapping</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A18" s="23" t="str">
+        <x:v>LL-TOPO</x:v>
+      </x:c>
+      <x:c r="B18" s="23" t="str">
+        <x:v>loss_landscape</x:v>
+      </x:c>
+      <x:c r="C18" s="23" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D18" s="23" t="str">
+        <x:v>conditional</x:v>
+      </x:c>
+      <x:c r="E18" s="23" t="str">
+        <x:v>Do sampled sublevel sets contain robust topological features?</x:v>
+      </x:c>
+      <x:c r="F18" s="23" t="str">
+        <x:v>persistent homology on a low-dimensional sampled surface</x:v>
+      </x:c>
+      <x:c r="G18" s="23" t="str">
+        <x:v>sampling-density convergence | multiple subspaces</x:v>
+      </x:c>
+      <x:c r="H18" s="23" t="str">
+        <x:v>mode-connectivity ambiguity remains</x:v>
+      </x:c>
+      <x:c r="I18" s="23" t="str"/>
+      <x:c r="J18" s="23" t="str">
+        <x:v>topology of a slice is not topology of full parameter space</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="23" t="str">
+        <x:v>LL-MEP</x:v>
+      </x:c>
+      <x:c r="B19" s="23" t="str">
+        <x:v>loss_landscape</x:v>
+      </x:c>
+      <x:c r="C19" s="23" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="str">
+        <x:v>conditional</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="str">
+        <x:v>What barrier separates two fixed minima?</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="str">
+        <x:v>approximate minimum-energy path or string method</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="str">
+        <x:v>known endpoints | path discretization convergence</x:v>
+      </x:c>
+      <x:c r="H19" s="23" t="str">
+        <x:v>linear interpolation shows a reproducible barrier</x:v>
+      </x:c>
+      <x:c r="I19" s="23" t="str">
+        <x:v>OP-01</x:v>
+      </x:c>
+      <x:c r="J19" s="23" t="str">
+        <x:v>computationally expensive and path-dependent</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:J1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="52" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="42" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="42" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="42" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="42" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="42" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
+      <x:c r="A1" s="17" t="str">
+        <x:v>Primary-source evidence register</x:v>
+      </x:c>
+      <x:c r="B1" s="17"/>
+      <x:c r="C1" s="17"/>
+      <x:c r="D1" s="17"/>
+      <x:c r="E1" s="17"/>
+      <x:c r="F1" s="17"/>
+      <x:c r="G1" s="17"/>
+      <x:c r="H1" s="17"/>
+      <x:c r="I1" s="17"/>
+      <x:c r="J1" s="17"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="18"/>
+      <x:c r="B2" s="18"/>
+      <x:c r="C2" s="18"/>
+      <x:c r="D2" s="18"/>
+      <x:c r="E2" s="18"/>
+      <x:c r="F2" s="18"/>
+      <x:c r="G2" s="18"/>
+      <x:c r="H2" s="18"/>
+      <x:c r="I2" s="18"/>
+      <x:c r="J2" s="18"/>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="22" t="str">
+        <x:v>evidence_id</x:v>
+      </x:c>
+      <x:c r="B3" s="22" t="str">
+        <x:v>experiment_id</x:v>
+      </x:c>
+      <x:c r="C3" s="22" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="D3" s="22" t="str">
+        <x:v>primary_source</x:v>
+      </x:c>
+      <x:c r="E3" s="22" t="str">
+        <x:v>year</x:v>
+      </x:c>
+      <x:c r="F3" s="22" t="str">
+        <x:v>architecture_or_method</x:v>
+      </x:c>
+      <x:c r="G3" s="22" t="str">
+        <x:v>claimed_mechanism</x:v>
+      </x:c>
+      <x:c r="H3" s="22" t="str">
+        <x:v>transfer_prediction</x:v>
+      </x:c>
+      <x:c r="I3" s="22" t="str">
+        <x:v>important_difference</x:v>
+      </x:c>
+      <x:c r="J3" s="22" t="str">
+        <x:v>decision_after_result</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A4" s="23" t="str">
+        <x:v>RQA-1987</x:v>
+      </x:c>
+      <x:c r="B4" s="23" t="str">
+        <x:v>FA-00</x:v>
+      </x:c>
+      <x:c r="C4" s="23" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="D4" s="23" t="str">
+        <x:v>https://doi.org/10.1209/0295-5075/4/9/004</x:v>
+      </x:c>
+      <x:c r="E4" s="23" t="str">
+        <x:v>1987</x:v>
+      </x:c>
+      <x:c r="F4" s="23" t="str">
+        <x:v>recurrence plot</x:v>
+      </x:c>
+      <x:c r="G4" s="23" t="str">
+        <x:v>visualizes recurrences of dynamical trajectories</x:v>
+      </x:c>
+      <x:c r="H4" s="23" t="str">
+        <x:v>teacher and surrogate should share recurrence structure</x:v>
+      </x:c>
+      <x:c r="I4" s="23" t="str">
+        <x:v>observed coordinates are not a proved minimal embedding</x:v>
+      </x:c>
+      <x:c r="J4" s="23" t="str">
+        <x:v>retained_as_diagnostic</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A5" s="23" t="str">
+        <x:v>LL-2018</x:v>
+      </x:c>
+      <x:c r="B5" s="23" t="str">
+        <x:v>DG-01</x:v>
+      </x:c>
+      <x:c r="C5" s="23" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2018/hash/a41b3bb3e6b050b6c9067c67f663b915-Abstract.html</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="str">
+        <x:v>2018</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="str">
+        <x:v>filter-normalized landscape visualization</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="str">
+        <x:v>makes perturbation directions more comparable</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="str">
+        <x:v>regime losses may have distinguishable local geometry</x:v>
+      </x:c>
+      <x:c r="I5" s="23" t="str">
+        <x:v>slices remain parameterization- and direction-dependent</x:v>
+      </x:c>
+      <x:c r="J5" s="23" t="str">
+        <x:v>preregistered</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A6" s="23" t="str">
+        <x:v>HESS-2017</x:v>
+      </x:c>
+      <x:c r="B6" s="23" t="str">
+        <x:v>DG-01</x:v>
+      </x:c>
+      <x:c r="C6" s="23" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="str">
+        <x:v>https://arxiv.org/abs/1611.07476</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="str">
+        <x:v>2017</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="str">
+        <x:v>Hessian eigenspectrum analysis</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="str">
+        <x:v>relates large-batch generalization and sharp directions</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="str">
+        <x:v>top eigenvalues and trace can distinguish local curvature</x:v>
+      </x:c>
+      <x:c r="I6" s="23" t="str">
+        <x:v>curvature is local and parameterization-dependent</x:v>
+      </x:c>
+      <x:c r="J6" s="23" t="str">
+        <x:v>preregistered</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A7" s="23" t="str">
+        <x:v>PCGRAD-2020</x:v>
+      </x:c>
+      <x:c r="B7" s="23" t="str">
+        <x:v>DG-01;LO-04</x:v>
+      </x:c>
+      <x:c r="C7" s="23" t="str">
+        <x:v>watch</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="str">
+        <x:v>https://arxiv.org/abs/2001.06782</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="str">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="str">
+        <x:v>gradient surgery</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="str">
+        <x:v>projects conflicting task gradients</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="str">
+        <x:v>use only if state-family gradients show stable negative cosine</x:v>
+      </x:c>
+      <x:c r="I7" s="23" t="str">
+        <x:v>state families are losses over one physical task not independent tasks</x:v>
+      </x:c>
+      <x:c r="J7" s="23" t="str">
+        <x:v>await_diagnosis</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="23" t="str">
+        <x:v>WN-2016</x:v>
+      </x:c>
+      <x:c r="B8" s="23" t="str">
+        <x:v>SC-01;SC-02</x:v>
+      </x:c>
+      <x:c r="C8" s="23" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="str">
+        <x:v>https://arxiv.org/abs/1609.03499</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="str">
+        <x:v>2016</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="str">
+        <x:v>dilated causal Conv1d</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="str">
+        <x:v>expands temporal receptive field efficiently</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="str">
+        <x:v>frontend may expose short multiscale patterns</x:v>
+      </x:c>
+      <x:c r="I8" s="23" t="str">
+        <x:v>our composition is not a WaveNet stack</x:v>
+      </x:c>
+      <x:c r="J8" s="23" t="str">
+        <x:v>scoped_rejection_for_7_5ms_frontend</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A9" s="23" t="str">
+        <x:v>GRU-2014</x:v>
+      </x:c>
+      <x:c r="B9" s="23" t="str">
+        <x:v>SC-01;SR-01</x:v>
+      </x:c>
+      <x:c r="C9" s="23" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="str">
+        <x:v>https://arxiv.org/abs/1412.3555</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="str">
+        <x:v>2014</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="str">
+        <x:v>GRU</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="str">
+        <x:v>gated causal sequence memory</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="str">
+        <x:v>strong smooth-dynamics baseline and state-feedback control</x:v>
+      </x:c>
+      <x:c r="I9" s="23" t="str">
+        <x:v>paper does not establish the Hay composition</x:v>
+      </x:c>
+      <x:c r="J9" s="23" t="str">
+        <x:v>baseline_retained</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A10" s="23" t="str">
+        <x:v>LSTM-1997</x:v>
+      </x:c>
+      <x:c r="B10" s="23" t="str">
+        <x:v>SC-02</x:v>
+      </x:c>
+      <x:c r="C10" s="23" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="D10" s="23" t="str">
+        <x:v>https://doi.org/10.1162/neco.1997.9.8.1735</x:v>
+      </x:c>
+      <x:c r="E10" s="23" t="str">
+        <x:v>1997</x:v>
+      </x:c>
+      <x:c r="F10" s="23" t="str">
+        <x:v>LSTM</x:v>
+      </x:c>
+      <x:c r="G10" s="23" t="str">
+        <x:v>separate gated cell state supports long credit assignment</x:v>
+      </x:c>
+      <x:c r="H10" s="23" t="str">
+        <x:v>may preserve slow state while handling fast input</x:v>
+      </x:c>
+      <x:c r="I10" s="23" t="str">
+        <x:v>fixed-dt continuous trajectories have no natural sequence reset</x:v>
+      </x:c>
+      <x:c r="J10" s="23" t="str">
+        <x:v>planned_capability_screen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A11" s="23" t="str">
+        <x:v>CFC-2022</x:v>
+      </x:c>
+      <x:c r="B11" s="23" t="str">
+        <x:v>SC-03</x:v>
+      </x:c>
+      <x:c r="C11" s="23" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="str">
+        <x:v>https://doi.org/10.1038/s42256-022-00556-7</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="str">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="str">
+        <x:v>CfC</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="str">
+        <x:v>closed-form explicit-time continuous recurrent dynamics</x:v>
+      </x:c>
+      <x:c r="H11" s="23" t="str">
+        <x:v>may represent mixed timescales efficiently</x:v>
+      </x:c>
+      <x:c r="I11" s="23" t="str">
+        <x:v>fixed dt exercises only part of the continuous-time benefit</x:v>
+      </x:c>
+      <x:c r="J11" s="23" t="str">
+        <x:v>planned_capability_screen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="23" t="str">
+        <x:v>LTC-2021</x:v>
+      </x:c>
+      <x:c r="B12" s="23" t="str">
+        <x:v>SC-04</x:v>
+      </x:c>
+      <x:c r="C12" s="23" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="str">
+        <x:v>https://doi.org/10.1609/aaai.v35i9.16936</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="str">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="str">
+        <x:v>LTC</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="str">
+        <x:v>state/input-dependent time constants</x:v>
+      </x:c>
+      <x:c r="H12" s="23" t="str">
+        <x:v>may allocate distinct effective timescales</x:v>
+      </x:c>
+      <x:c r="I12" s="23" t="str">
+        <x:v>solver settings and cost confound comparisons</x:v>
+      </x:c>
+      <x:c r="J12" s="23" t="str">
+        <x:v>planned_capability_screen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="23" t="str">
+        <x:v>SAM-2020</x:v>
+      </x:c>
+      <x:c r="B13" s="23" t="str">
+        <x:v>RG-01;OP-01</x:v>
+      </x:c>
+      <x:c r="C13" s="23" t="str">
+        <x:v>watch</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="str">
+        <x:v>https://arxiv.org/abs/2010.01412</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="str">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="str">
+        <x:v>sharpness-aware minimization</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="str">
+        <x:v>optimizes neighborhood sharpness</x:v>
+      </x:c>
+      <x:c r="H13" s="23" t="str">
+        <x:v>test only if sharpness and instability are measured</x:v>
+      </x:c>
+      <x:c r="I13" s="23" t="str">
+        <x:v>not specific to dynamical rollout and doubles work</x:v>
+      </x:c>
+      <x:c r="J13" s="23" t="str">
+        <x:v>blocked_by_DG_01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="23" t="str">
+        <x:v>SWA-2018</x:v>
+      </x:c>
+      <x:c r="B14" s="23" t="str">
+        <x:v>OP-01</x:v>
+      </x:c>
+      <x:c r="C14" s="23" t="str">
+        <x:v>watch</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="str">
+        <x:v>https://arxiv.org/abs/1803.05407</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="str">
+        <x:v>2018</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="str">
+        <x:v>stochastic weight averaging</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="str">
+        <x:v>averages weights along an optimization trajectory</x:v>
+      </x:c>
+      <x:c r="H14" s="23" t="str">
+        <x:v>may improve a connected flat basin</x:v>
+      </x:c>
+      <x:c r="I14" s="23" t="str">
+        <x:v>cannot repair missing representation or event exposure</x:v>
+      </x:c>
+      <x:c r="J14" s="23" t="str">
+        <x:v>blocked_by_DG_01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A15" s="23" t="str">
+        <x:v>MRSTFT-2019</x:v>
+      </x:c>
+      <x:c r="B15" s="23" t="str">
+        <x:v>LO-01;INT-01</x:v>
+      </x:c>
+      <x:c r="C15" s="23" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="str">
+        <x:v>https://arxiv.org/abs/1910.11480</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="str">
+        <x:v>2019</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="str">
+        <x:v>multi-resolution STFT loss</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="str">
+        <x:v>matches time-frequency magnitude at several resolutions</x:v>
+      </x:c>
+      <x:c r="H15" s="23" t="str">
+        <x:v>should penalize high-frequency collapse</x:v>
+      </x:c>
+      <x:c r="I15" s="23" t="str">
+        <x:v>audio source domain and no event-amplitude guarantee</x:v>
+      </x:c>
+      <x:c r="J15" s="23" t="str">
+        <x:v>helpful_slow_but_insufficient_for_spikes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="23" t="str">
+        <x:v>STFT-2018</x:v>
+      </x:c>
+      <x:c r="B16" s="23" t="str">
+        <x:v>LO-01</x:v>
+      </x:c>
+      <x:c r="C16" s="23" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="str">
+        <x:v>https://arxiv.org/abs/1810.11945</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="str">
+        <x:v>2018</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="str">
+        <x:v>STFT spectral loss</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="str">
+        <x:v>differentiable spectral waveform objective</x:v>
+      </x:c>
+      <x:c r="H16" s="23" t="str">
+        <x:v>can restore broadband trajectories with MSE</x:v>
+      </x:c>
+      <x:c r="I16" s="23" t="str">
+        <x:v>magnitude terms may ignore exact phase</x:v>
+      </x:c>
+      <x:c r="J16" s="23" t="str">
+        <x:v>insufficient_for_spikes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A17" s="23" t="str">
+        <x:v>BMSE-2022</x:v>
+      </x:c>
+      <x:c r="B17" s="23" t="str">
+        <x:v>TR-01;LO-02</x:v>
+      </x:c>
+      <x:c r="C17" s="23" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2022/html/Ren_Balanced_MSE_for_Imbalanced_Visual_Regression_CVPR_2022_paper.html</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="str">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="F17" s="23" t="str">
+        <x:v>Balanced MSE</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="str">
+        <x:v>corrects target-density imbalance in continuous regression</x:v>
+      </x:c>
+      <x:c r="H17" s="23" t="str">
+        <x:v>may reduce conditional-mean collapse of rare voltage extremes</x:v>
+      </x:c>
+      <x:c r="I17" s="23" t="str">
+        <x:v>vision setting and target density is multivariate/time-dependent here</x:v>
+      </x:c>
+      <x:c r="J17" s="23" t="str">
+        <x:v>await_DG_01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="23" t="str">
+        <x:v>TCN-2018</x:v>
+      </x:c>
+      <x:c r="B18" s="23" t="str">
+        <x:v>CB-01</x:v>
+      </x:c>
+      <x:c r="C18" s="23" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="D18" s="23" t="str">
+        <x:v>https://arxiv.org/abs/1803.01271</x:v>
+      </x:c>
+      <x:c r="E18" s="23" t="str">
+        <x:v>2018</x:v>
+      </x:c>
+      <x:c r="F18" s="23" t="str">
+        <x:v>temporal convolutional network</x:v>
+      </x:c>
+      <x:c r="G18" s="23" t="str">
+        <x:v>finite causal receptive field with residual convolutions</x:v>
+      </x:c>
+      <x:c r="H18" s="23" t="str">
+        <x:v>tests local event localization without recurrent state</x:v>
+      </x:c>
+      <x:c r="I18" s="23" t="str">
+        <x:v>full Hay dynamics may exceed a fixed receptive field</x:v>
+      </x:c>
+      <x:c r="J18" s="23" t="str">
+        <x:v>planned_capability_screen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A19" s="23" t="str">
+        <x:v>S4-2021</x:v>
+      </x:c>
+      <x:c r="B19" s="23" t="str">
+        <x:v>CB-01;SC-05</x:v>
+      </x:c>
+      <x:c r="C19" s="23" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="str">
+        <x:v>https://arxiv.org/abs/2111.00396</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="str">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="str">
+        <x:v>S4</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="str">
+        <x:v>structured state-space long convolution</x:v>
+      </x:c>
+      <x:c r="H19" s="23" t="str">
+        <x:v>may preserve long memory and stable fast-slow responses</x:v>
+      </x:c>
+      <x:c r="I19" s="23" t="str">
+        <x:v>original tasks differ and implementation complexity must be controlled</x:v>
+      </x:c>
+      <x:c r="J19" s="23" t="str">
+        <x:v>planned_capability_screen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="23" t="str">
+        <x:v>MAMBA-2023</x:v>
+      </x:c>
+      <x:c r="B20" s="23" t="str">
+        <x:v>SC-07</x:v>
+      </x:c>
+      <x:c r="C20" s="23" t="str">
+        <x:v>watch</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="str">
+        <x:v>https://arxiv.org/abs/2312.00752</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="str">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="str">
+        <x:v>selective state-space model</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="str">
+        <x:v>input-dependent state-space selection</x:v>
+      </x:c>
+      <x:c r="H20" s="23" t="str">
+        <x:v>may help only if content-dependent selection is missing</x:v>
+      </x:c>
+      <x:c r="I20" s="23" t="str">
+        <x:v>larger modern implementation can confound capacity</x:v>
+      </x:c>
+      <x:c r="J20" s="23" t="str">
+        <x:v>conditional_after_S4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A21" s="23" t="str">
+        <x:v>NODE-2018</x:v>
+      </x:c>
+      <x:c r="B21" s="23" t="str">
+        <x:v>SC-06</x:v>
+      </x:c>
+      <x:c r="C21" s="23" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="D21" s="23" t="str">
+        <x:v>https://proceedings.neurips.cc/paper/2018/hash/69386f6bb1dfed68692a24c8686939b9-Abstract.html</x:v>
+      </x:c>
+      <x:c r="E21" s="23" t="str">
+        <x:v>2018</x:v>
+      </x:c>
+      <x:c r="F21" s="23" t="str">
+        <x:v>Neural ODE</x:v>
+      </x:c>
+      <x:c r="G21" s="23" t="str">
+        <x:v>learned vector field integrated continuously</x:v>
+      </x:c>
+      <x:c r="H21" s="23" t="str">
+        <x:v>matches a physical-state flow prior</x:v>
+      </x:c>
+      <x:c r="I21" s="23" t="str">
+        <x:v>spike inputs are discontinuous controls and solver cost matters</x:v>
+      </x:c>
+      <x:c r="J21" s="23" t="str">
+        <x:v>planned_with_explicit_control_contract</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A22" s="23" t="str">
+        <x:v>NCDE-2020</x:v>
+      </x:c>
+      <x:c r="B22" s="23" t="str">
+        <x:v>SC-06</x:v>
+      </x:c>
+      <x:c r="C22" s="23" t="str">
+        <x:v>watch</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="str">
+        <x:v>https://proceedings.neurips.cc/paper/2020/hash/4a5876b450b45371f6cfe5047ac8cd45-Abstract.html</x:v>
+      </x:c>
+      <x:c r="E22" s="23" t="str">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="F22" s="23" t="str">
+        <x:v>Neural CDE</x:v>
+      </x:c>
+      <x:c r="G22" s="23" t="str">
+        <x:v>hidden dynamics driven by a control path</x:v>
+      </x:c>
+      <x:c r="H22" s="23" t="str">
+        <x:v>useful if irregular timing or continuous controls enter the task</x:v>
+      </x:c>
+      <x:c r="I22" s="23" t="str">
+        <x:v>current fixed-dt binary event bins weaken its unique advantage</x:v>
+      </x:c>
+      <x:c r="J22" s="23" t="str">
+        <x:v>conditional</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A23" s="23" t="str">
+        <x:v>MPNN-2017</x:v>
+      </x:c>
+      <x:c r="B23" s="23" t="str">
+        <x:v>CB-02;SP-01</x:v>
+      </x:c>
+      <x:c r="C23" s="23" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="D23" s="23" t="str">
+        <x:v>https://proceedings.mlr.press/v70/gilmer17a.html</x:v>
+      </x:c>
+      <x:c r="E23" s="23" t="str">
+        <x:v>2017</x:v>
+      </x:c>
+      <x:c r="F23" s="23" t="str">
+        <x:v>message-passing neural network</x:v>
+      </x:c>
+      <x:c r="G23" s="23" t="str">
+        <x:v>shared node updates and edge messages</x:v>
+      </x:c>
+      <x:c r="H23" s="23" t="str">
+        <x:v>matches four-compartment local coupling</x:v>
+      </x:c>
+      <x:c r="I23" s="23" t="str">
+        <x:v>fixed known morphology is tiny and monolithic capacity control is essential</x:v>
+      </x:c>
+      <x:c r="J23" s="23" t="str">
+        <x:v>planned_capability_screen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A24" s="23" t="str">
+        <x:v>MOE-2017</x:v>
+      </x:c>
+      <x:c r="B24" s="23" t="str">
+        <x:v>HY-01</x:v>
+      </x:c>
+      <x:c r="C24" s="23" t="str">
+        <x:v>watch</x:v>
+      </x:c>
+      <x:c r="D24" s="23" t="str">
+        <x:v>https://arxiv.org/abs/1701.06538</x:v>
+      </x:c>
+      <x:c r="E24" s="23" t="str">
+        <x:v>2017</x:v>
+      </x:c>
+      <x:c r="F24" s="23" t="str">
+        <x:v>sparse mixture of experts</x:v>
+      </x:c>
+      <x:c r="G24" s="23" t="str">
+        <x:v>conditional specialized computation</x:v>
+      </x:c>
+      <x:c r="H24" s="23" t="str">
+        <x:v>may separate rare transition and common regimes</x:v>
+      </x:c>
+      <x:c r="I24" s="23" t="str">
+        <x:v>previous router success did not imply a capable correction expert</x:v>
+      </x:c>
+      <x:c r="J24" s="23" t="str">
+        <x:v>blocked_until_expert_capability</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A25" s="23" t="str">
+        <x:v>CW-RNN-2014</x:v>
+      </x:c>
+      <x:c r="B25" s="23" t="str">
+        <x:v>HY-02</x:v>
+      </x:c>
+      <x:c r="C25" s="23" t="str">
+        <x:v>watch</x:v>
+      </x:c>
+      <x:c r="D25" s="23" t="str">
+        <x:v>https://arxiv.org/abs/1402.3511</x:v>
+      </x:c>
+      <x:c r="E25" s="23" t="str">
+        <x:v>2014</x:v>
+      </x:c>
+      <x:c r="F25" s="23" t="str">
+        <x:v>clockwork recurrent neural network</x:v>
+      </x:c>
+      <x:c r="G25" s="23" t="str">
+        <x:v>modules update at distinct periods</x:v>
+      </x:c>
+      <x:c r="H25" s="23" t="str">
+        <x:v>may reflect measured slow-fast separation</x:v>
+      </x:c>
+      <x:c r="I25" s="23" t="str">
+        <x:v>hard periods may mismatch state-dependent biological timescales</x:v>
+      </x:c>
+      <x:c r="J25" s="23" t="str">
+        <x:v>conditional</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:J1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -4985,31 +7292,21 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="8" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="40" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="42" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="28" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="46" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="52" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="32" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="85" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
       <x:c r="A1" s="17" t="str">
-        <x:v>Diagnostic and intervention catalog</x:v>
+        <x:v>Full architecture taxonomy by inductive bias</x:v>
       </x:c>
       <x:c r="B1" s="17"/>
       <x:c r="C1" s="17"/>
       <x:c r="D1" s="17"/>
       <x:c r="E1" s="17"/>
-      <x:c r="F1" s="17"/>
-      <x:c r="G1" s="17"/>
-      <x:c r="H1" s="17"/>
-      <x:c r="I1" s="17"/>
-      <x:c r="J1" s="17"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="18"/>
@@ -5017,555 +7314,486 @@
       <x:c r="C2" s="18"/>
       <x:c r="D2" s="18"/>
       <x:c r="E2" s="18"/>
-      <x:c r="F2" s="18"/>
-      <x:c r="G2" s="18"/>
-      <x:c r="H2" s="18"/>
-      <x:c r="I2" s="18"/>
-      <x:c r="J2" s="18"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="22" t="str">
-        <x:v>ID</x:v>
+        <x:v>Level</x:v>
       </x:c>
       <x:c r="B3" s="22" t="str">
-        <x:v>Category</x:v>
+        <x:v>Level name</x:v>
       </x:c>
       <x:c r="C3" s="22" t="str">
-        <x:v>Tier</x:v>
+        <x:v>Assumption</x:v>
       </x:c>
       <x:c r="D3" s="22" t="str">
-        <x:v>Status</x:v>
+        <x:v>Family</x:v>
       </x:c>
       <x:c r="E3" s="22" t="str">
-        <x:v>Question</x:v>
-      </x:c>
-      <x:c r="F3" s="22" t="str">
-        <x:v>Method</x:v>
-      </x:c>
-      <x:c r="G3" s="22" t="str">
-        <x:v>Controls</x:v>
-      </x:c>
-      <x:c r="H3" s="22" t="str">
-        <x:v>Trigger</x:v>
-      </x:c>
-      <x:c r="I3" s="22" t="str">
-        <x:v>Authorized interventions</x:v>
-      </x:c>
-      <x:c r="J3" s="22" t="str">
-        <x:v>Interpretation limits</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A4" s="23" t="str">
-        <x:v>OUT-EVENT</x:v>
+        <x:v>Members</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="23" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B4" s="23" t="str">
-        <x:v>output</x:v>
-      </x:c>
-      <x:c r="C4" s="23" t="n">
+        <x:v>universal foundations</x:v>
+      </x:c>
+      <x:c r="C4" s="23" t="str">
+        <x:v>the datum can be treated as a vector or distribution</x:v>
+      </x:c>
+      <x:c r="D4" s="23" t="str">
+        <x:v>pure feed-forward</x:v>
+      </x:c>
+      <x:c r="E4" s="23" t="str">
+        <x:v>MLP; Radial Basis Function Network; KAN; MLP-Mixer; gMLP; ResMLP</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A5" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B5" s="23" t="str">
+        <x:v>universal foundations</x:v>
+      </x:c>
+      <x:c r="C5" s="23" t="str">
+        <x:v>the datum can be treated as a vector or distribution</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="str">
+        <x:v>representation by reconstruction</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="str">
+        <x:v>vanilla autoencoder; denoising autoencoder; sparse autoencoder; contractive autoencoder; VAE; beta-VAE; Wasserstein AE; VQ-VAE; masked autoencoder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B6" s="23" t="str">
+        <x:v>universal foundations</x:v>
+      </x:c>
+      <x:c r="C6" s="23" t="str">
+        <x:v>the datum can be treated as a vector or distribution</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="str">
+        <x:v>energy and equilibrium</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="str">
+        <x:v>classical Hopfield network; modern Hopfield network; RBM; DBN; DBM; Helmholtz machine; generic EBM</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B7" s="23" t="str">
+        <x:v>universal foundations</x:v>
+      </x:c>
+      <x:c r="C7" s="23" t="str">
+        <x:v>the datum can be treated as a vector or distribution</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="str">
+        <x:v>reservoir computing</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="str">
+        <x:v>Echo State Network; Liquid State Machine</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B8" s="23" t="str">
+        <x:v>universal foundations</x:v>
+      </x:c>
+      <x:c r="C8" s="23" t="str">
+        <x:v>the datum can be treated as a vector or distribution</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="str">
+        <x:v>probabilistic uncertainty</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="str">
+        <x:v>Bayesian neural network; Deep Gaussian Process; Neural Process; Conditional Neural Process</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A9" s="23" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D4" s="23" t="str">
-        <x:v>active</x:v>
-      </x:c>
-      <x:c r="E4" s="23" t="str">
-        <x:v>Are rare transitions recovered in amplitude, timing and count?</x:v>
-      </x:c>
-      <x:c r="F4" s="23" t="str">
-        <x:v>precision/recall/F1, peak error, event-window RMSE and phase error</x:v>
-      </x:c>
-      <x:c r="G4" s="23" t="str">
-        <x:v>fixed threshold | tolerance sweep | teacher event count</x:v>
-      </x:c>
-      <x:c r="H4" s="23" t="str">
-        <x:v>zero recall or amplitude compression</x:v>
-      </x:c>
-      <x:c r="I4" s="23" t="str">
-        <x:v>DG-01; TR-01; LO-02; SR-01</x:v>
-      </x:c>
-      <x:c r="J4" s="23" t="str">
-        <x:v>threshold metrics alone do not measure subthreshold fidelity</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A5" s="23" t="str">
-        <x:v>OUT-ROLL</x:v>
-      </x:c>
-      <x:c r="B5" s="23" t="str">
-        <x:v>output</x:v>
-      </x:c>
-      <x:c r="C5" s="23" t="n">
+      <x:c r="B9" s="23" t="str">
+        <x:v>weak structural bias</x:v>
+      </x:c>
+      <x:c r="C9" s="23" t="str">
+        <x:v>generic symmetries, relations, metric structure or external memory exist without a fixed task topology</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="str">
+        <x:v>equivariance and symmetry</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="str">
+        <x:v>G-CNN; steerable CNN; E(n)-equivariant GNN; SE(3)-Transformer; Tensor Field Network; Lie Group Network; gauge-equivariant CNN; capsule network; geometric deep learning</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A10" s="23" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D5" s="23" t="str">
-        <x:v>active</x:v>
-      </x:c>
-      <x:c r="E5" s="23" t="str">
-        <x:v>How does error grow under closed-loop rollout?</x:v>
-      </x:c>
-      <x:c r="F5" s="23" t="str">
-        <x:v>horizon-conditioned NRMSE and first-threshold-crossing divergence</x:v>
-      </x:c>
-      <x:c r="G5" s="23" t="str">
-        <x:v>same initial context | no teacher forcing after initialization</x:v>
-      </x:c>
-      <x:c r="H5" s="23" t="str">
-        <x:v>superlinear drift or family-specific divergence</x:v>
-      </x:c>
-      <x:c r="I5" s="23" t="str">
-        <x:v>SR-01; LO-03</x:v>
-      </x:c>
-      <x:c r="J5" s="23" t="str">
-        <x:v>finite horizons are task definitions, not universal stability proofs</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A6" s="23" t="str">
-        <x:v>LL-INTERP</x:v>
-      </x:c>
-      <x:c r="B6" s="23" t="str">
-        <x:v>loss_landscape</x:v>
-      </x:c>
-      <x:c r="C6" s="23" t="n">
+      <x:c r="B10" s="23" t="str">
+        <x:v>weak structural bias</x:v>
+      </x:c>
+      <x:c r="C10" s="23" t="str">
+        <x:v>generic symmetries, relations, metric structure or external memory exist without a fixed task topology</x:v>
+      </x:c>
+      <x:c r="D10" s="23" t="str">
+        <x:v>generic relational attention</x:v>
+      </x:c>
+      <x:c r="E10" s="23" t="str">
+        <x:v>Transformer; multi-head self-attention; cross-attention; linear attention; sparse attention; Reformer; Performer; Nyströmformer; Perceiver; Perceiver IO; Set Transformer; ISAB; Slot Attention</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A11" s="23" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D6" s="23" t="str">
-        <x:v>preregistered</x:v>
-      </x:c>
-      <x:c r="E6" s="23" t="str">
-        <x:v>Does training cross a barrier into a smooth low-frequency basin?</x:v>
-      </x:c>
-      <x:c r="F6" s="23" t="str">
-        <x:v>loss along filter-normalized initial-to-final and paired-checkpoint interpolation</x:v>
-      </x:c>
-      <x:c r="G6" s="23" t="str">
-        <x:v>frozen validation batches by regime | BatchNorm statistics frozen | no test data</x:v>
-      </x:c>
-      <x:c r="H6" s="23" t="str">
-        <x:v>event loss barrier absent from common-regime loss</x:v>
-      </x:c>
-      <x:c r="I6" s="23" t="str">
-        <x:v>OP-01; LO-02</x:v>
-      </x:c>
-      <x:c r="J6" s="23" t="str">
-        <x:v>a 1-D path is not the full landscape</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A7" s="23" t="str">
-        <x:v>LL-SLICE</x:v>
-      </x:c>
-      <x:c r="B7" s="23" t="str">
-        <x:v>loss_landscape</x:v>
-      </x:c>
-      <x:c r="C7" s="23" t="n">
+      <x:c r="B11" s="23" t="str">
+        <x:v>weak structural bias</x:v>
+      </x:c>
+      <x:c r="C11" s="23" t="str">
+        <x:v>generic symmetries, relations, metric structure or external memory exist without a fixed task topology</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="str">
+        <x:v>metric learning</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="str">
+        <x:v>Siamese network; triplet network; prototypical network; SimCLR pattern; MoCo pattern; BYOL pattern</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A12" s="23" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D7" s="23" t="str">
-        <x:v>preregistered</x:v>
-      </x:c>
-      <x:c r="E7" s="23" t="str">
-        <x:v>Are local neighborhoods sharp, anisotropic or regime-dependent?</x:v>
-      </x:c>
-      <x:c r="F7" s="23" t="str">
-        <x:v>filter-normalized 1-D/2-D random-direction slices</x:v>
-      </x:c>
-      <x:c r="G7" s="23" t="str">
-        <x:v>same perturbation radii | multiple direction seeds | parameter-group report</x:v>
-      </x:c>
-      <x:c r="H7" s="23" t="str">
-        <x:v>event curvature differs strongly from global curvature</x:v>
-      </x:c>
-      <x:c r="I7" s="23" t="str">
-        <x:v>RG-01; OP-01</x:v>
-      </x:c>
-      <x:c r="J7" s="23" t="str">
-        <x:v>visual roughness depends on direction sampling</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A8" s="23" t="str">
-        <x:v>LL-HESS-TOP</x:v>
-      </x:c>
-      <x:c r="B8" s="23" t="str">
-        <x:v>loss_landscape</x:v>
-      </x:c>
-      <x:c r="C8" s="23" t="n">
+      <x:c r="B12" s="23" t="str">
+        <x:v>weak structural bias</x:v>
+      </x:c>
+      <x:c r="C12" s="23" t="str">
+        <x:v>generic symmetries, relations, metric structure or external memory exist without a fixed task topology</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="str">
+        <x:v>external differentiable memory</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="str">
+        <x:v>Neural Turing Machine; Differentiable Neural Computer; Memory Network; End-to-End Memory Network; memory-augmented neural network</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A13" s="23" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D8" s="23" t="str">
-        <x:v>preregistered</x:v>
-      </x:c>
-      <x:c r="E8" s="23" t="str">
-        <x:v>What is the strongest local curvature?</x:v>
-      </x:c>
-      <x:c r="F8" s="23" t="str">
-        <x:v>Hessian-vector products with power iteration/Lanczos</x:v>
-      </x:c>
-      <x:c r="G8" s="23" t="str">
-        <x:v>same frozen batches | convergence residual | parameter normalization</x:v>
-      </x:c>
-      <x:c r="H8" s="23" t="str">
-        <x:v>large event-conditioned eigenvalue or scaffold-specific curvature spike</x:v>
-      </x:c>
-      <x:c r="I8" s="23" t="str">
-        <x:v>OP-01; RG-01</x:v>
-      </x:c>
-      <x:c r="J8" s="23" t="str">
-        <x:v>largest eigenvalue omits most directions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="23" t="str">
-        <x:v>LL-HESS-TRACE</x:v>
-      </x:c>
-      <x:c r="B9" s="23" t="str">
-        <x:v>loss_landscape</x:v>
-      </x:c>
-      <x:c r="C9" s="23" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D9" s="23" t="str">
-        <x:v>preregistered</x:v>
-      </x:c>
-      <x:c r="E9" s="23" t="str">
-        <x:v>How much aggregate curvature is present?</x:v>
-      </x:c>
-      <x:c r="F9" s="23" t="str">
-        <x:v>Hutchinson trace estimate with confidence interval</x:v>
-      </x:c>
-      <x:c r="G9" s="23" t="str">
-        <x:v>fixed probe seeds | probe-count convergence</x:v>
-      </x:c>
-      <x:c r="H9" s="23" t="str">
-        <x:v>large trace with high anisotropy</x:v>
-      </x:c>
-      <x:c r="I9" s="23" t="str">
-        <x:v>OP-01; RG-01</x:v>
-      </x:c>
-      <x:c r="J9" s="23" t="str">
-        <x:v>stochastic estimator and parameterization dependent</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A10" s="23" t="str">
-        <x:v>GR-CONFLICT</x:v>
-      </x:c>
-      <x:c r="B10" s="23" t="str">
-        <x:v>gradient</x:v>
-      </x:c>
-      <x:c r="C10" s="23" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D10" s="23" t="str">
-        <x:v>preregistered</x:v>
-      </x:c>
-      <x:c r="E10" s="23" t="str">
-        <x:v>Do event, subthreshold, slow and synaptic objectives request opposing updates?</x:v>
-      </x:c>
-      <x:c r="F10" s="23" t="str">
-        <x:v>pairwise gradient cosine matrix by parameter block</x:v>
-      </x:c>
-      <x:c r="G10" s="23" t="str">
-        <x:v>identical examples | loss-scale normalized companion view | bootstrap intervals</x:v>
-      </x:c>
-      <x:c r="H10" s="23" t="str">
-        <x:v>stable negative cosine or extreme norm imbalance</x:v>
-      </x:c>
-      <x:c r="I10" s="23" t="str">
-        <x:v>LO-02; LO-04; TR-01</x:v>
-      </x:c>
-      <x:c r="J10" s="23" t="str">
-        <x:v>local conflicts do not prove global incompatibility</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A11" s="23" t="str">
-        <x:v>GR-SNR</x:v>
-      </x:c>
-      <x:c r="B11" s="23" t="str">
-        <x:v>gradient</x:v>
-      </x:c>
-      <x:c r="C11" s="23" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D11" s="23" t="str">
-        <x:v>preregistered</x:v>
-      </x:c>
-      <x:c r="E11" s="23" t="str">
-        <x:v>Is the rare-event gradient visible above minibatch noise?</x:v>
-      </x:c>
-      <x:c r="F11" s="23" t="str">
-        <x:v>per-regime gradient norm, variance and signal-to-noise ratio</x:v>
-      </x:c>
-      <x:c r="G11" s="23" t="str">
-        <x:v>equal example counts | multiple minibatches</x:v>
-      </x:c>
-      <x:c r="H11" s="23" t="str">
-        <x:v>event gradient SNR low or contribution negligible</x:v>
-      </x:c>
-      <x:c r="I11" s="23" t="str">
-        <x:v>TR-01; LO-02</x:v>
-      </x:c>
-      <x:c r="J11" s="23" t="str">
-        <x:v>estimator depends on batching</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A12" s="23" t="str">
-        <x:v>ACT-SEP</x:v>
-      </x:c>
-      <x:c r="B12" s="23" t="str">
-        <x:v>activation</x:v>
-      </x:c>
-      <x:c r="C12" s="23" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D12" s="23" t="str">
-        <x:v>planned</x:v>
-      </x:c>
-      <x:c r="E12" s="23" t="str">
-        <x:v>Where does event/non-event separability appear and disappear?</x:v>
-      </x:c>
-      <x:c r="F12" s="23" t="str">
-        <x:v>linear probes and distribution distances per layer/time lag</x:v>
-      </x:c>
-      <x:c r="G12" s="23" t="str">
-        <x:v>held-out validation trajectories | probe capacity fixed</x:v>
-      </x:c>
-      <x:c r="H12" s="23" t="str">
-        <x:v>early separability followed by readout collapse</x:v>
-      </x:c>
-      <x:c r="I12" s="23" t="str">
-        <x:v>SR-01; HY-01</x:v>
-      </x:c>
-      <x:c r="J12" s="23" t="str">
-        <x:v>decodability is not causal use</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="15" hidden="0" customHeight="1">
-      <x:c r="A13" s="23" t="str">
-        <x:v>ACT-SAT</x:v>
-      </x:c>
       <x:c r="B13" s="23" t="str">
-        <x:v>activation</x:v>
-      </x:c>
-      <x:c r="C13" s="23" t="n">
-        <x:v>1</x:v>
+        <x:v>weak structural bias</x:v>
+      </x:c>
+      <x:c r="C13" s="23" t="str">
+        <x:v>generic symmetries, relations, metric structure or external memory exist without a fixed task topology</x:v>
       </x:c>
       <x:c r="D13" s="23" t="str">
-        <x:v>planned</x:v>
+        <x:v>state-space sequence operators</x:v>
       </x:c>
       <x:c r="E13" s="23" t="str">
-        <x:v>Do nonlinearities or gates saturate in the failed regime?</x:v>
-      </x:c>
-      <x:c r="F13" s="23" t="str">
-        <x:v>quantiles, dead/saturated fraction, gate entropy and derivatives</x:v>
-      </x:c>
-      <x:c r="G13" s="23" t="str">
-        <x:v>regime conditioning | same checkpoints</x:v>
-      </x:c>
-      <x:c r="H13" s="23" t="str">
-        <x:v>event-specific saturation with gradient attenuation</x:v>
-      </x:c>
-      <x:c r="I13" s="23" t="str">
-        <x:v>AC-01; NM-01</x:v>
-      </x:c>
-      <x:c r="J13" s="23" t="str">
-        <x:v>saturation may be adaptive rather than pathological</x:v>
+        <x:v>generic SSM; S4; S4D; S5; Mamba; Mamba-2; H3; Hyena; RWKV; RetNet; Griffin; xLSTM</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A14" s="23" t="str">
-        <x:v>ACT-RANK</x:v>
+      <x:c r="A14" s="23" t="n">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B14" s="23" t="str">
-        <x:v>activation</x:v>
-      </x:c>
-      <x:c r="C14" s="23" t="n">
-        <x:v>1</x:v>
+        <x:v>temporal bias</x:v>
+      </x:c>
+      <x:c r="C14" s="23" t="str">
+        <x:v>order, causality and/or physical timing matter</x:v>
       </x:c>
       <x:c r="D14" s="23" t="str">
-        <x:v>planned</x:v>
+        <x:v>discrete recurrence</x:v>
       </x:c>
       <x:c r="E14" s="23" t="str">
-        <x:v>Does the latent collapse to a low-dimensional smooth manifold?</x:v>
-      </x:c>
-      <x:c r="F14" s="23" t="str">
-        <x:v>effective rank, participation ratio and singular spectrum by regime</x:v>
-      </x:c>
-      <x:c r="G14" s="23" t="str">
-        <x:v>center/scale conventions | matched sample count</x:v>
-      </x:c>
-      <x:c r="H14" s="23" t="str">
-        <x:v>event trajectories require directions absent in prediction latent</x:v>
-      </x:c>
-      <x:c r="I14" s="23" t="str">
-        <x:v>SC-05; SR-01</x:v>
-      </x:c>
-      <x:c r="J14" s="23" t="str">
-        <x:v>rank depends on coordinate scaling</x:v>
+        <x:v>vanilla RNN; LSTM; GRU; bidirectional RNN; Clockwork RNN; Hierarchical Multiscale RNN; unitary RNN; orthogonal RNN; Quasi-RNN; SRU</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A15" s="23" t="str">
-        <x:v>DYN-RQA</x:v>
+      <x:c r="A15" s="23" t="n">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B15" s="23" t="str">
-        <x:v>dynamics</x:v>
-      </x:c>
-      <x:c r="C15" s="23" t="n">
-        <x:v>1</x:v>
+        <x:v>temporal bias</x:v>
+      </x:c>
+      <x:c r="C15" s="23" t="str">
+        <x:v>order, causality and/or physical timing matter</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
-        <x:v>active</x:v>
+        <x:v>continuous-time recurrence</x:v>
       </x:c>
       <x:c r="E15" s="23" t="str">
-        <x:v>Does the surrogate preserve recurrent dynamical structure?</x:v>
-      </x:c>
-      <x:c r="F15" s="23" t="str">
-        <x:v>recurrence plots, recurrence rate, determinism and laminarity</x:v>
-      </x:c>
-      <x:c r="G15" s="23" t="str">
-        <x:v>shared embedding rule | threshold sensitivity</x:v>
-      </x:c>
-      <x:c r="H15" s="23" t="str">
-        <x:v>regime-specific topology mismatch</x:v>
-      </x:c>
-      <x:c r="I15" s="23" t="str">
-        <x:v>SC-05; SC-06</x:v>
-      </x:c>
-      <x:c r="J15" s="23" t="str">
-        <x:v>Takens-style reconstruction assumptions must be stated</x:v>
+        <x:v>Neural ODE; Augmented Neural ODE; Neural CDE; Neural SDE; Liquid Time-Constant network; CTRNN; Latent ODE; ODE-RNN</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A16" s="23" t="str">
-        <x:v>LL-MODE</x:v>
+      <x:c r="A16" s="23" t="n">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B16" s="23" t="str">
-        <x:v>loss_landscape</x:v>
-      </x:c>
-      <x:c r="C16" s="23" t="n">
+        <x:v>temporal bias</x:v>
+      </x:c>
+      <x:c r="C16" s="23" t="str">
+        <x:v>order, causality and/or physical timing matter</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="str">
+        <x:v>event-driven timing</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="str">
+        <x:v>Neural Point Process; Temporal Point Process; Neural Hawkes Process; continuous-time event model; asynchronous timestamp model</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A17" s="23" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D16" s="23" t="str">
-        <x:v>conditional</x:v>
-      </x:c>
-      <x:c r="E16" s="23" t="str">
-        <x:v>Are independently trained solutions connected by low-loss paths?</x:v>
-      </x:c>
-      <x:c r="F16" s="23" t="str">
-        <x:v>linear and polygonal mode connectivity</x:v>
-      </x:c>
-      <x:c r="G16" s="23" t="str">
-        <x:v>permutation alignment | same data and objective</x:v>
-      </x:c>
-      <x:c r="H16" s="23" t="str">
-        <x:v>seed instability plus distinct basins in Tier 1</x:v>
-      </x:c>
-      <x:c r="I16" s="23" t="str">
-        <x:v>OP-01</x:v>
-      </x:c>
-      <x:c r="J16" s="23" t="str">
-        <x:v>connectivity can change under symmetry alignment</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A17" s="23" t="str">
-        <x:v>LL-FRACTAL</x:v>
-      </x:c>
       <x:c r="B17" s="23" t="str">
-        <x:v>loss_landscape</x:v>
-      </x:c>
-      <x:c r="C17" s="23" t="n">
+        <x:v>temporal bias</x:v>
+      </x:c>
+      <x:c r="C17" s="23" t="str">
+        <x:v>order, causality and/or physical timing matter</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="str">
+        <x:v>attention over sequences</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="str">
+        <x:v>Bahdanau attention; Luong attention; autoregressive Transformer; bidirectional Transformer; encoder-decoder Transformer; Transformer-XL; Compressive Transformer; Universal Transformer; Adaptive Computation Time</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="23" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D17" s="23" t="str">
-        <x:v>conditional</x:v>
-      </x:c>
-      <x:c r="E17" s="23" t="str">
-        <x:v>Is apparent roughness scale-dependent?</x:v>
-      </x:c>
-      <x:c r="F17" s="23" t="str">
-        <x:v>wavelet spectrum, Hölder/fractal or multifractal estimators on controlled slices</x:v>
-      </x:c>
-      <x:c r="G17" s="23" t="str">
-        <x:v>large scale range | synthetic calibration surfaces | uncertainty</x:v>
-      </x:c>
-      <x:c r="H17" s="23" t="str">
-        <x:v>unresolved multi-scale roughness after Tier 1</x:v>
-      </x:c>
-      <x:c r="I17" s="23" t="str"/>
-      <x:c r="J17" s="23" t="str">
-        <x:v>high estimator variance and weak direct intervention mapping</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A18" s="23" t="str">
-        <x:v>LL-TOPO</x:v>
-      </x:c>
       <x:c r="B18" s="23" t="str">
-        <x:v>loss_landscape</x:v>
-      </x:c>
-      <x:c r="C18" s="23" t="n">
-        <x:v>2</x:v>
+        <x:v>temporal bias</x:v>
+      </x:c>
+      <x:c r="C18" s="23" t="str">
+        <x:v>order, causality and/or physical timing matter</x:v>
       </x:c>
       <x:c r="D18" s="23" t="str">
-        <x:v>conditional</x:v>
+        <x:v>explicit position and time encoding</x:v>
       </x:c>
       <x:c r="E18" s="23" t="str">
-        <x:v>Do sampled sublevel sets contain robust topological features?</x:v>
-      </x:c>
-      <x:c r="F18" s="23" t="str">
-        <x:v>persistent homology on a low-dimensional sampled surface</x:v>
-      </x:c>
-      <x:c r="G18" s="23" t="str">
-        <x:v>sampling-density convergence | multiple subspaces</x:v>
-      </x:c>
-      <x:c r="H18" s="23" t="str">
-        <x:v>mode-connectivity ambiguity remains</x:v>
-      </x:c>
-      <x:c r="I18" s="23" t="str"/>
-      <x:c r="J18" s="23" t="str">
-        <x:v>topology of a slice is not topology of full parameter space</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="15" hidden="0" customHeight="1">
-      <x:c r="A19" s="23" t="str">
-        <x:v>LL-MEP</x:v>
+        <x:v>sinusoidal position; learned position; relative position; RoPE; ALiBi; CoPE; T5 relative bias</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A19" s="23" t="n">
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B19" s="23" t="str">
-        <x:v>loss_landscape</x:v>
-      </x:c>
-      <x:c r="C19" s="23" t="n">
-        <x:v>2</x:v>
+        <x:v>spatial and multiscale bias</x:v>
+      </x:c>
+      <x:c r="C19" s="23" t="str">
+        <x:v>locality, translation structure, spatial hierarchy or explicit resolution bands exist</x:v>
       </x:c>
       <x:c r="D19" s="23" t="str">
-        <x:v>conditional</x:v>
+        <x:v>atomic convolution operators</x:v>
       </x:c>
       <x:c r="E19" s="23" t="str">
-        <x:v>What barrier separates two fixed minima?</x:v>
-      </x:c>
-      <x:c r="F19" s="23" t="str">
-        <x:v>approximate minimum-energy path or string method</x:v>
-      </x:c>
-      <x:c r="G19" s="23" t="str">
-        <x:v>known endpoints | path discretization convergence</x:v>
-      </x:c>
-      <x:c r="H19" s="23" t="str">
-        <x:v>linear interpolation shows a reproducible barrier</x:v>
-      </x:c>
-      <x:c r="I19" s="23" t="str">
-        <x:v>OP-01</x:v>
-      </x:c>
-      <x:c r="J19" s="23" t="str">
-        <x:v>computationally expensive and path-dependent</x:v>
+        <x:v>standard convolution; depthwise convolution; depthwise-separable convolution; grouped convolution; dilated convolution; deformable convolution; transposed convolution; 1x1 channel mixing; 3D convolution; 2+1D convolution; dynamic convolution; conditional convolution</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A20" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B20" s="23" t="str">
+        <x:v>spatial and multiscale bias</x:v>
+      </x:c>
+      <x:c r="C20" s="23" t="str">
+        <x:v>locality, translation structure, spatial hierarchy or explicit resolution bands exist</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="str">
+        <x:v>foundational CNNs</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="str">
+        <x:v>LeNet; AlexNet; VGG; Inception; ResNet; ResNeXt; DenseNet; Squeeze-and-Excitation; CBAM; ECA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A21" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B21" s="23" t="str">
+        <x:v>spatial and multiscale bias</x:v>
+      </x:c>
+      <x:c r="C21" s="23" t="str">
+        <x:v>locality, translation structure, spatial hierarchy or explicit resolution bands exist</x:v>
+      </x:c>
+      <x:c r="D21" s="23" t="str">
+        <x:v>efficient CNNs</x:v>
+      </x:c>
+      <x:c r="E21" s="23" t="str">
+        <x:v>MobileNet; ShuffleNet; SqueezeNet; GhostNet; EfficientNet</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A22" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B22" s="23" t="str">
+        <x:v>spatial and multiscale bias</x:v>
+      </x:c>
+      <x:c r="C22" s="23" t="str">
+        <x:v>locality, translation structure, spatial hierarchy or explicit resolution bands exist</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="str">
+        <x:v>modern CNNs</x:v>
+      </x:c>
+      <x:c r="E22" s="23" t="str">
+        <x:v>ConvNeXt; RepVGG; SLaK; UniRepLKNet; FocalNet; HorNet</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A23" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B23" s="23" t="str">
+        <x:v>spatial and multiscale bias</x:v>
+      </x:c>
+      <x:c r="C23" s="23" t="str">
+        <x:v>locality, translation structure, spatial hierarchy or explicit resolution bands exist</x:v>
+      </x:c>
+      <x:c r="D23" s="23" t="str">
+        <x:v>vision transformer hybrids</x:v>
+      </x:c>
+      <x:c r="E23" s="23" t="str">
+        <x:v>ViT; DeiT; BEiT; Swin Transformer; CoAtNet; MaxViT; CvT; MetaFormer; PoolFormer</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A24" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B24" s="23" t="str">
+        <x:v>spatial and multiscale bias</x:v>
+      </x:c>
+      <x:c r="C24" s="23" t="str">
+        <x:v>locality, translation structure, spatial hierarchy or explicit resolution bands exist</x:v>
+      </x:c>
+      <x:c r="D24" s="23" t="str">
+        <x:v>explicit feature pyramids</x:v>
+      </x:c>
+      <x:c r="E24" s="23" t="str">
+        <x:v>FPN; PANet; BiFPN; NAS-FPN; ASPP</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A25" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B25" s="23" t="str">
+        <x:v>spatial and multiscale bias</x:v>
+      </x:c>
+      <x:c r="C25" s="23" t="str">
+        <x:v>locality, translation structure, spatial hierarchy or explicit resolution bands exist</x:v>
+      </x:c>
+      <x:c r="D25" s="23" t="str">
+        <x:v>frequency and multiresolution</x:v>
+      </x:c>
+      <x:c r="E25" s="23" t="str">
+        <x:v>scattering network; wavelet neural network; multi-resolution analysis network</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A26" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B26" s="23" t="str">
+        <x:v>relational and topological bias</x:v>
+      </x:c>
+      <x:c r="C26" s="23" t="str">
+        <x:v>the system has an explicit graph, hierarchy, combinatorial structure or non-Euclidean geometry</x:v>
+      </x:c>
+      <x:c r="D26" s="23" t="str">
+        <x:v>message passing on graphs</x:v>
+      </x:c>
+      <x:c r="E26" s="23" t="str">
+        <x:v>GCN; GraphSAGE; GAT; GIN; MPNN; ChebNet; DiffPool; TopKPool; MinCutPool</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A27" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B27" s="23" t="str">
+        <x:v>relational and topological bias</x:v>
+      </x:c>
+      <x:c r="C27" s="23" t="str">
+        <x:v>the system has an explicit graph, hierarchy, combinatorial structure or non-Euclidean geometry</x:v>
+      </x:c>
+      <x:c r="D27" s="23" t="str">
+        <x:v>dynamic and higher-order graphs</x:v>
+      </x:c>
+      <x:c r="E27" s="23" t="str">
+        <x:v>Temporal Graph Network; hypergraph neural network; simplicial neural network; cellular neural network; sheaf neural network</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A28" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B28" s="23" t="str">
+        <x:v>relational and topological bias</x:v>
+      </x:c>
+      <x:c r="C28" s="23" t="str">
+        <x:v>the system has an explicit graph, hierarchy, combinatorial structure or non-Euclidean geometry</x:v>
+      </x:c>
+      <x:c r="D28" s="23" t="str">
+        <x:v>combinatorial structures</x:v>
+      </x:c>
+      <x:c r="E28" s="23" t="str">
+        <x:v>recursive neural network; Tree-LSTM; Tree-GRU; DAG network; algebraic-structure network</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A29" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B29" s="23" t="str">
+        <x:v>relational and topological bias</x:v>
+      </x:c>
+      <x:c r="C29" s="23" t="str">
+        <x:v>the system has an explicit graph, hierarchy, combinatorial structure or non-Euclidean geometry</x:v>
+      </x:c>
+      <x:c r="D29" s="23" t="str">
+        <x:v>non-Euclidean geometry</x:v>
+      </x:c>
+      <x:c r="E29" s="23" t="str">
+        <x:v>hyperbolic neural network; Poincaré embedding; Lorentzian model; mixed-curvature product space</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A30" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B30" s="23" t="str">
+        <x:v>relational and topological bias</x:v>
+      </x:c>
+      <x:c r="C30" s="23" t="str">
+        <x:v>the system has an explicit graph, hierarchy, combinatorial structure or non-Euclidean geometry</x:v>
+      </x:c>
+      <x:c r="D30" s="23" t="str">
+        <x:v>explicit relational inference</x:v>
+      </x:c>
+      <x:c r="E30" s="23" t="str">
+        <x:v>Relation Network; Interaction Network; Neural Relational Inference; Relational Memory Core</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:J1"/>
+    <x:mergeCell ref="A1:E1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -5575,21 +7803,18 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="52" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="42" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="42" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="42" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="42" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="42" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="55" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="55" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="45" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
       <x:c r="A1" s="17" t="str">
-        <x:v>Primary-source evidence register</x:v>
+        <x:v>Functional design-pattern library</x:v>
       </x:c>
       <x:c r="B1" s="17"/>
       <x:c r="C1" s="17"/>
@@ -5597,9 +7822,6 @@
       <x:c r="E1" s="17"/>
       <x:c r="F1" s="17"/>
       <x:c r="G1" s="17"/>
-      <x:c r="H1" s="17"/>
-      <x:c r="I1" s="17"/>
-      <x:c r="J1" s="17"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="18"/>
@@ -5609,749 +7831,309 @@
       <x:c r="E2" s="18"/>
       <x:c r="F2" s="18"/>
       <x:c r="G2" s="18"/>
-      <x:c r="H2" s="18"/>
-      <x:c r="I2" s="18"/>
-      <x:c r="J2" s="18"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="22" t="str">
-        <x:v>evidence_id</x:v>
+        <x:v>ID</x:v>
       </x:c>
       <x:c r="B3" s="22" t="str">
-        <x:v>experiment_id</x:v>
+        <x:v>Class</x:v>
       </x:c>
       <x:c r="C3" s="22" t="str">
-        <x:v>status</x:v>
+        <x:v>Pattern</x:v>
       </x:c>
       <x:c r="D3" s="22" t="str">
-        <x:v>primary_source</x:v>
+        <x:v>Functional hypothesis</x:v>
       </x:c>
       <x:c r="E3" s="22" t="str">
-        <x:v>year</x:v>
+        <x:v>Diagnostic trigger</x:v>
       </x:c>
       <x:c r="F3" s="22" t="str">
-        <x:v>architecture_or_method</x:v>
+        <x:v>Required tests</x:v>
       </x:c>
       <x:c r="G3" s="22" t="str">
-        <x:v>claimed_mechanism</x:v>
-      </x:c>
-      <x:c r="H3" s="22" t="str">
-        <x:v>transfer_prediction</x:v>
-      </x:c>
-      <x:c r="I3" s="22" t="str">
-        <x:v>important_difference</x:v>
-      </x:c>
-      <x:c r="J3" s="22" t="str">
-        <x:v>decision_after_result</x:v>
+        <x:v>Sources</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A4" s="23" t="str">
-        <x:v>RQA-1987</x:v>
+        <x:v>PAT-RESIDUAL</x:v>
       </x:c>
       <x:c r="B4" s="23" t="str">
-        <x:v>FA-00</x:v>
+        <x:v>information flow</x:v>
       </x:c>
       <x:c r="C4" s="23" t="str">
-        <x:v>accepted</x:v>
+        <x:v>residual/skip path</x:v>
       </x:c>
       <x:c r="D4" s="23" t="str">
-        <x:v>https://doi.org/10.1209/0295-5075/4/9/004</x:v>
+        <x:v>preserve an easier representation and improve backward feature correction</x:v>
       </x:c>
       <x:c r="E4" s="23" t="str">
-        <x:v>1987</x:v>
+        <x:v>useful early feature exists but degrades with depth or gradient flow</x:v>
       </x:c>
       <x:c r="F4" s="23" t="str">
-        <x:v>recurrence plot</x:v>
+        <x:v>layerwise probe; ablation; gradient by depth</x:v>
       </x:c>
       <x:c r="G4" s="23" t="str">
-        <x:v>visualizes recurrences of dynamical trajectories</x:v>
-      </x:c>
-      <x:c r="H4" s="23" t="str">
-        <x:v>teacher and surrogate should share recurrence structure</x:v>
-      </x:c>
-      <x:c r="I4" s="23" t="str">
-        <x:v>observed coordinates are not a proved minimal embedding</x:v>
-      </x:c>
-      <x:c r="J4" s="23" t="str">
-        <x:v>retained_as_diagnostic</x:v>
+        <x:v>SRC-POLM-4-1B; SRC-POLM-4-2</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A5" s="23" t="str">
-        <x:v>LL-2018</x:v>
+        <x:v>PAT-HORIZONTAL</x:v>
       </x:c>
       <x:c r="B5" s="23" t="str">
-        <x:v>DG-01</x:v>
+        <x:v>information flow</x:v>
       </x:c>
       <x:c r="C5" s="23" t="str">
-        <x:v>accepted</x:v>
+        <x:v>local horizontal causal mixing</x:v>
       </x:c>
       <x:c r="D5" s="23" t="str">
-        <x:v>https://proceedings.neurips.cc/paper_files/paper/2018/hash/a41b3bb3e6b050b6c9067c67f663b915-Abstract.html</x:v>
+        <x:v>make short-range neighboring information directly accessible without burdening the global mechanism</x:v>
       </x:c>
       <x:c r="E5" s="23" t="str">
-        <x:v>2018</x:v>
+        <x:v>required local context is present but expensive/inaccessible at the readout</x:v>
       </x:c>
       <x:c r="F5" s="23" t="str">
-        <x:v>filter-normalized landscape visualization</x:v>
+        <x:v>receptive-field microtask; insertion-point ablation; locality-length sweep</x:v>
       </x:c>
       <x:c r="G5" s="23" t="str">
-        <x:v>makes perturbation directions more comparable</x:v>
-      </x:c>
-      <x:c r="H5" s="23" t="str">
-        <x:v>regime losses may have distinguishable local geometry</x:v>
-      </x:c>
-      <x:c r="I5" s="23" t="str">
-        <x:v>slices remain parameterization- and direction-dependent</x:v>
-      </x:c>
-      <x:c r="J5" s="23" t="str">
-        <x:v>preregistered</x:v>
+        <x:v>SRC-POLM-4-1B; SRC-POLM-4-2</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A6" s="23" t="str">
-        <x:v>HESS-2017</x:v>
+        <x:v>PAT-GATING</x:v>
       </x:c>
       <x:c r="B6" s="23" t="str">
-        <x:v>DG-01</x:v>
+        <x:v>conditional dynamics</x:v>
       </x:c>
       <x:c r="C6" s="23" t="str">
-        <x:v>accepted</x:v>
+        <x:v>standard gated update</x:v>
       </x:c>
       <x:c r="D6" s="23" t="str">
-        <x:v>https://arxiv.org/abs/1611.07476</x:v>
+        <x:v>learn input/state-dependent retention and overwrite</x:v>
       </x:c>
       <x:c r="E6" s="23" t="str">
-        <x:v>2017</x:v>
+        <x:v>different regimes require different memory retention</x:v>
       </x:c>
       <x:c r="F6" s="23" t="str">
-        <x:v>Hessian eigenspectrum analysis</x:v>
+        <x:v>gate trajectory analysis; fixed-gate control; timescale microtask</x:v>
       </x:c>
       <x:c r="G6" s="23" t="str">
-        <x:v>relates large-batch generalization and sharp directions</x:v>
-      </x:c>
-      <x:c r="H6" s="23" t="str">
-        <x:v>top eigenvalues and trace can distinguish local curvature</x:v>
-      </x:c>
-      <x:c r="I6" s="23" t="str">
-        <x:v>curvature is local and parameterization-dependent</x:v>
-      </x:c>
-      <x:c r="J6" s="23" t="str">
-        <x:v>preregistered</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>SRC-TAXONOMY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="23" t="str">
-        <x:v>PCGRAD-2020</x:v>
+        <x:v>PAT-MULTIRATE</x:v>
       </x:c>
       <x:c r="B7" s="23" t="str">
-        <x:v>DG-01;LO-04</x:v>
+        <x:v>temporal hierarchy</x:v>
       </x:c>
       <x:c r="C7" s="23" t="str">
-        <x:v>watch</x:v>
+        <x:v>explicit multirate modules</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
-        <x:v>https://arxiv.org/abs/2001.06782</x:v>
+        <x:v>separate updates with distinct characteristic timescales</x:v>
       </x:c>
       <x:c r="E7" s="23" t="str">
-        <x:v>2020</x:v>
+        <x:v>state families show reproducible timescale-separated drift</x:v>
       </x:c>
       <x:c r="F7" s="23" t="str">
-        <x:v>gradient surgery</x:v>
+        <x:v>delay surface; rate ablation; matched-update control</x:v>
       </x:c>
       <x:c r="G7" s="23" t="str">
-        <x:v>projects conflicting task gradients</x:v>
-      </x:c>
-      <x:c r="H7" s="23" t="str">
-        <x:v>use only if state-family gradients show stable negative cosine</x:v>
-      </x:c>
-      <x:c r="I7" s="23" t="str">
-        <x:v>state families are losses over one physical task not independent tasks</x:v>
-      </x:c>
-      <x:c r="J7" s="23" t="str">
-        <x:v>await_diagnosis</x:v>
+        <x:v>SRC-TAXONOMY; SRC-CREATIVE</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="23" t="str">
-        <x:v>WN-2016</x:v>
+        <x:v>PAT-STATE-FEEDBACK</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str">
-        <x:v>SC-01;SC-02</x:v>
+        <x:v>information contract</x:v>
       </x:c>
       <x:c r="C8" s="23" t="str">
-        <x:v>accepted</x:v>
+        <x:v>own predicted-state feedback</x:v>
       </x:c>
       <x:c r="D8" s="23" t="str">
-        <x:v>https://arxiv.org/abs/1609.03499</x:v>
+        <x:v>make a physical Markov summary explicit</x:v>
       </x:c>
       <x:c r="E8" s="23" t="str">
-        <x:v>2016</x:v>
+        <x:v>latent contains broad regime but exact phase/state is inaccessible</x:v>
       </x:c>
       <x:c r="F8" s="23" t="str">
-        <x:v>dilated causal Conv1d</x:v>
+        <x:v>input-only control; teacher-leak audit; closed-loop horizon</x:v>
       </x:c>
       <x:c r="G8" s="23" t="str">
-        <x:v>expands temporal receptive field efficiently</x:v>
-      </x:c>
-      <x:c r="H8" s="23" t="str">
-        <x:v>frontend may expose short multiscale patterns</x:v>
-      </x:c>
-      <x:c r="I8" s="23" t="str">
-        <x:v>our composition is not a WaveNet stack</x:v>
-      </x:c>
-      <x:c r="J8" s="23" t="str">
-        <x:v>scoped_rejection_for_7_5ms_frontend</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>SRC-SYSID-LANDSCAPE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="23" t="str">
-        <x:v>GRU-2014</x:v>
+        <x:v>PAT-SSM</x:v>
       </x:c>
       <x:c r="B9" s="23" t="str">
-        <x:v>SC-01;SR-01</x:v>
+        <x:v>sequence operator</x:v>
       </x:c>
       <x:c r="C9" s="23" t="str">
-        <x:v>accepted</x:v>
+        <x:v>structured state-space memory</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
-        <x:v>https://arxiv.org/abs/1412.3555</x:v>
+        <x:v>represent stable long kernels and fast-slow responses efficiently</x:v>
       </x:c>
       <x:c r="E9" s="23" t="str">
-        <x:v>2014</x:v>
+        <x:v>long memory and stable propagation fail under recurrence</x:v>
       </x:c>
       <x:c r="F9" s="23" t="str">
-        <x:v>GRU</x:v>
+        <x:v>capacity x delay surface; impulse response; spectral analysis</x:v>
       </x:c>
       <x:c r="G9" s="23" t="str">
-        <x:v>gated causal sequence memory</x:v>
-      </x:c>
-      <x:c r="H9" s="23" t="str">
-        <x:v>strong smooth-dynamics baseline and state-feedback control</x:v>
-      </x:c>
-      <x:c r="I9" s="23" t="str">
-        <x:v>paper does not establish the Hay composition</x:v>
-      </x:c>
-      <x:c r="J9" s="23" t="str">
-        <x:v>baseline_retained</x:v>
+        <x:v>SRC-TAXONOMY</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A10" s="23" t="str">
-        <x:v>LSTM-1997</x:v>
+        <x:v>PAT-CONTINUOUS</x:v>
       </x:c>
       <x:c r="B10" s="23" t="str">
-        <x:v>SC-02</x:v>
+        <x:v>continuous dynamics</x:v>
       </x:c>
       <x:c r="C10" s="23" t="str">
-        <x:v>accepted</x:v>
+        <x:v>continuous-time recurrent/vector-field operator</x:v>
       </x:c>
       <x:c r="D10" s="23" t="str">
-        <x:v>https://doi.org/10.1162/neco.1997.9.8.1735</x:v>
+        <x:v>encode continuous flow and explicit timing</x:v>
       </x:c>
       <x:c r="E10" s="23" t="str">
-        <x:v>1997</x:v>
+        <x:v>fixed-step scaffold shows timescale or irregular-timing failure</x:v>
       </x:c>
       <x:c r="F10" s="23" t="str">
-        <x:v>LSTM</x:v>
+        <x:v>dt generalization; solver/tolerance control; event-jump handling</x:v>
       </x:c>
       <x:c r="G10" s="23" t="str">
-        <x:v>separate gated cell state supports long credit assignment</x:v>
-      </x:c>
-      <x:c r="H10" s="23" t="str">
-        <x:v>may preserve slow state while handling fast input</x:v>
-      </x:c>
-      <x:c r="I10" s="23" t="str">
-        <x:v>fixed-dt continuous trajectories have no natural sequence reset</x:v>
-      </x:c>
-      <x:c r="J10" s="23" t="str">
-        <x:v>planned_capability_screen</x:v>
+        <x:v>SRC-TAXONOMY</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A11" s="23" t="str">
-        <x:v>CFC-2022</x:v>
+        <x:v>PAT-MESSAGE</x:v>
       </x:c>
       <x:c r="B11" s="23" t="str">
-        <x:v>SC-03</x:v>
+        <x:v>spatial topology</x:v>
       </x:c>
       <x:c r="C11" s="23" t="str">
-        <x:v>accepted</x:v>
+        <x:v>shared local message passing</x:v>
       </x:c>
       <x:c r="D11" s="23" t="str">
-        <x:v>https://doi.org/10.1038/s42256-022-00556-7</x:v>
+        <x:v>factor local compartment updates from edge-mediated coupling</x:v>
       </x:c>
       <x:c r="E11" s="23" t="str">
-        <x:v>2022</x:v>
+        <x:v>errors follow compartment distance or source-target structure</x:v>
       </x:c>
       <x:c r="F11" s="23" t="str">
-        <x:v>CfC</x:v>
+        <x:v>four-node propagation; edge ablation; monolithic parameter control</x:v>
       </x:c>
       <x:c r="G11" s="23" t="str">
-        <x:v>closed-form explicit-time continuous recurrent dynamics</x:v>
-      </x:c>
-      <x:c r="H11" s="23" t="str">
-        <x:v>may represent mixed timescales efficiently</x:v>
-      </x:c>
-      <x:c r="I11" s="23" t="str">
-        <x:v>fixed dt exercises only part of the continuous-time benefit</x:v>
-      </x:c>
-      <x:c r="J11" s="23" t="str">
-        <x:v>planned_capability_screen</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="15" hidden="0" customHeight="1">
+        <x:v>SRC-TAXONOMY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A12" s="23" t="str">
-        <x:v>LTC-2021</x:v>
+        <x:v>PAT-MOE</x:v>
       </x:c>
       <x:c r="B12" s="23" t="str">
-        <x:v>SC-04</x:v>
+        <x:v>regime specialization</x:v>
       </x:c>
       <x:c r="C12" s="23" t="str">
-        <x:v>accepted</x:v>
+        <x:v>mixture/switching experts</x:v>
       </x:c>
       <x:c r="D12" s="23" t="str">
-        <x:v>https://doi.org/10.1609/aaai.v35i9.16936</x:v>
+        <x:v>allocate specialized computation to separable dynamical regimes</x:v>
       </x:c>
       <x:c r="E12" s="23" t="str">
-        <x:v>2021</x:v>
+        <x:v>regime is causally separable and a specialized expert independently works</x:v>
       </x:c>
       <x:c r="F12" s="23" t="str">
-        <x:v>LTC</x:v>
+        <x:v>router calibration; oracle-router upper bound; expert capability; spill guardrail</x:v>
       </x:c>
       <x:c r="G12" s="23" t="str">
-        <x:v>state/input-dependent time constants</x:v>
-      </x:c>
-      <x:c r="H12" s="23" t="str">
-        <x:v>may allocate distinct effective timescales</x:v>
-      </x:c>
-      <x:c r="I12" s="23" t="str">
-        <x:v>solver settings and cost confound comparisons</x:v>
-      </x:c>
-      <x:c r="J12" s="23" t="str">
-        <x:v>planned_capability_screen</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="15" hidden="0" customHeight="1">
+        <x:v>SRC-TAXONOMY; SRC-CREATIVE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A13" s="23" t="str">
-        <x:v>SAM-2020</x:v>
+        <x:v>PAT-MULTIRES</x:v>
       </x:c>
       <x:c r="B13" s="23" t="str">
-        <x:v>RG-01;OP-01</x:v>
+        <x:v>scale decomposition</x:v>
       </x:c>
       <x:c r="C13" s="23" t="str">
-        <x:v>watch</x:v>
+        <x:v>wavelet or multiresolution path</x:v>
       </x:c>
       <x:c r="D13" s="23" t="str">
-        <x:v>https://arxiv.org/abs/2010.01412</x:v>
+        <x:v>expose localized temporal/frequency scales</x:v>
       </x:c>
       <x:c r="E13" s="23" t="str">
-        <x:v>2020</x:v>
+        <x:v>errors are sharply scale-localized and spectral loss alone is insufficient</x:v>
       </x:c>
       <x:c r="F13" s="23" t="str">
-        <x:v>sharpness-aware minimization</x:v>
+        <x:v>scale ablation; phase-preserving control; reconstruction microtask</x:v>
       </x:c>
       <x:c r="G13" s="23" t="str">
-        <x:v>optimizes neighborhood sharpness</x:v>
-      </x:c>
-      <x:c r="H13" s="23" t="str">
-        <x:v>test only if sharpness and instability are measured</x:v>
-      </x:c>
-      <x:c r="I13" s="23" t="str">
-        <x:v>not specific to dynamical rollout and doubles work</x:v>
-      </x:c>
-      <x:c r="J13" s="23" t="str">
-        <x:v>blocked_by_DG_01</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="15" hidden="0" customHeight="1">
+        <x:v>SRC-TAXONOMY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A14" s="23" t="str">
-        <x:v>SWA-2018</x:v>
+        <x:v>PAT-MEMORY</x:v>
       </x:c>
       <x:c r="B14" s="23" t="str">
-        <x:v>OP-01</x:v>
+        <x:v>content-addressable memory</x:v>
       </x:c>
       <x:c r="C14" s="23" t="str">
-        <x:v>watch</x:v>
+        <x:v>external/attentive retrieval</x:v>
       </x:c>
       <x:c r="D14" s="23" t="str">
-        <x:v>https://arxiv.org/abs/1803.05407</x:v>
+        <x:v>retrieve a prior pattern by content rather than fixed delay</x:v>
       </x:c>
       <x:c r="E14" s="23" t="str">
-        <x:v>2018</x:v>
+        <x:v>long recurrence depends on similarity not elapsed time</x:v>
       </x:c>
       <x:c r="F14" s="23" t="str">
-        <x:v>stochastic weight averaging</x:v>
+        <x:v>repeat-with-variation microtask; memory ablation; retrieval precision</x:v>
       </x:c>
       <x:c r="G14" s="23" t="str">
-        <x:v>averages weights along an optimization trajectory</x:v>
-      </x:c>
-      <x:c r="H14" s="23" t="str">
-        <x:v>may improve a connected flat basin</x:v>
-      </x:c>
-      <x:c r="I14" s="23" t="str">
-        <x:v>cannot repair missing representation or event exposure</x:v>
-      </x:c>
-      <x:c r="J14" s="23" t="str">
-        <x:v>blocked_by_DG_01</x:v>
+        <x:v>SRC-TAXONOMY; SRC-CREATIVE</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A15" s="23" t="str">
-        <x:v>MRSTFT-2019</x:v>
+        <x:v>PAT-NORM</x:v>
       </x:c>
       <x:c r="B15" s="23" t="str">
-        <x:v>LO-01;INT-01</x:v>
+        <x:v>optimization geometry</x:v>
       </x:c>
       <x:c r="C15" s="23" t="str">
-        <x:v>accepted</x:v>
+        <x:v>normalization/scaling primitive</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
-        <x:v>https://arxiv.org/abs/1910.11480</x:v>
+        <x:v>condition feature and gradient scales</x:v>
       </x:c>
       <x:c r="E15" s="23" t="str">
-        <x:v>2019</x:v>
+        <x:v>measured activation or gradient scale pathology</x:v>
       </x:c>
       <x:c r="F15" s="23" t="str">
-        <x:v>multi-resolution STFT loss</x:v>
+        <x:v>invertible scaling control; single-normalizer ablation; Jacobian/gradient statistics</x:v>
       </x:c>
       <x:c r="G15" s="23" t="str">
-        <x:v>matches time-frequency magnitude at several resolutions</x:v>
-      </x:c>
-      <x:c r="H15" s="23" t="str">
-        <x:v>should penalize high-frequency collapse</x:v>
-      </x:c>
-      <x:c r="I15" s="23" t="str">
-        <x:v>audio source domain and no event-amplitude guarantee</x:v>
-      </x:c>
-      <x:c r="J15" s="23" t="str">
-        <x:v>helpful_slow_but_insufficient_for_spikes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="15" hidden="0" customHeight="1">
-      <x:c r="A16" s="23" t="str">
-        <x:v>STFT-2018</x:v>
-      </x:c>
-      <x:c r="B16" s="23" t="str">
-        <x:v>LO-01</x:v>
-      </x:c>
-      <x:c r="C16" s="23" t="str">
-        <x:v>accepted</x:v>
-      </x:c>
-      <x:c r="D16" s="23" t="str">
-        <x:v>https://arxiv.org/abs/1810.11945</x:v>
-      </x:c>
-      <x:c r="E16" s="23" t="str">
-        <x:v>2018</x:v>
-      </x:c>
-      <x:c r="F16" s="23" t="str">
-        <x:v>STFT spectral loss</x:v>
-      </x:c>
-      <x:c r="G16" s="23" t="str">
-        <x:v>differentiable spectral waveform objective</x:v>
-      </x:c>
-      <x:c r="H16" s="23" t="str">
-        <x:v>can restore broadband trajectories with MSE</x:v>
-      </x:c>
-      <x:c r="I16" s="23" t="str">
-        <x:v>magnitude terms may ignore exact phase</x:v>
-      </x:c>
-      <x:c r="J16" s="23" t="str">
-        <x:v>insufficient_for_spikes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A17" s="23" t="str">
-        <x:v>BMSE-2022</x:v>
-      </x:c>
-      <x:c r="B17" s="23" t="str">
-        <x:v>TR-01;LO-02</x:v>
-      </x:c>
-      <x:c r="C17" s="23" t="str">
-        <x:v>accepted</x:v>
-      </x:c>
-      <x:c r="D17" s="23" t="str">
-        <x:v>https://openaccess.thecvf.com/content/CVPR2022/html/Ren_Balanced_MSE_for_Imbalanced_Visual_Regression_CVPR_2022_paper.html</x:v>
-      </x:c>
-      <x:c r="E17" s="23" t="str">
-        <x:v>2022</x:v>
-      </x:c>
-      <x:c r="F17" s="23" t="str">
-        <x:v>Balanced MSE</x:v>
-      </x:c>
-      <x:c r="G17" s="23" t="str">
-        <x:v>corrects target-density imbalance in continuous regression</x:v>
-      </x:c>
-      <x:c r="H17" s="23" t="str">
-        <x:v>may reduce conditional-mean collapse of rare voltage extremes</x:v>
-      </x:c>
-      <x:c r="I17" s="23" t="str">
-        <x:v>vision setting and target density is multivariate/time-dependent here</x:v>
-      </x:c>
-      <x:c r="J17" s="23" t="str">
-        <x:v>await_DG_01</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="15" hidden="0" customHeight="1">
-      <x:c r="A18" s="23" t="str">
-        <x:v>TCN-2018</x:v>
-      </x:c>
-      <x:c r="B18" s="23" t="str">
-        <x:v>CB-01</x:v>
-      </x:c>
-      <x:c r="C18" s="23" t="str">
-        <x:v>accepted</x:v>
-      </x:c>
-      <x:c r="D18" s="23" t="str">
-        <x:v>https://arxiv.org/abs/1803.01271</x:v>
-      </x:c>
-      <x:c r="E18" s="23" t="str">
-        <x:v>2018</x:v>
-      </x:c>
-      <x:c r="F18" s="23" t="str">
-        <x:v>temporal convolutional network</x:v>
-      </x:c>
-      <x:c r="G18" s="23" t="str">
-        <x:v>finite causal receptive field with residual convolutions</x:v>
-      </x:c>
-      <x:c r="H18" s="23" t="str">
-        <x:v>tests local event localization without recurrent state</x:v>
-      </x:c>
-      <x:c r="I18" s="23" t="str">
-        <x:v>full Hay dynamics may exceed a fixed receptive field</x:v>
-      </x:c>
-      <x:c r="J18" s="23" t="str">
-        <x:v>planned_capability_screen</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A19" s="23" t="str">
-        <x:v>S4-2021</x:v>
-      </x:c>
-      <x:c r="B19" s="23" t="str">
-        <x:v>CB-01;SC-05</x:v>
-      </x:c>
-      <x:c r="C19" s="23" t="str">
-        <x:v>accepted</x:v>
-      </x:c>
-      <x:c r="D19" s="23" t="str">
-        <x:v>https://arxiv.org/abs/2111.00396</x:v>
-      </x:c>
-      <x:c r="E19" s="23" t="str">
-        <x:v>2021</x:v>
-      </x:c>
-      <x:c r="F19" s="23" t="str">
-        <x:v>S4</x:v>
-      </x:c>
-      <x:c r="G19" s="23" t="str">
-        <x:v>structured state-space long convolution</x:v>
-      </x:c>
-      <x:c r="H19" s="23" t="str">
-        <x:v>may preserve long memory and stable fast-slow responses</x:v>
-      </x:c>
-      <x:c r="I19" s="23" t="str">
-        <x:v>original tasks differ and implementation complexity must be controlled</x:v>
-      </x:c>
-      <x:c r="J19" s="23" t="str">
-        <x:v>planned_capability_screen</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="15" hidden="0" customHeight="1">
-      <x:c r="A20" s="23" t="str">
-        <x:v>MAMBA-2023</x:v>
-      </x:c>
-      <x:c r="B20" s="23" t="str">
-        <x:v>SC-07</x:v>
-      </x:c>
-      <x:c r="C20" s="23" t="str">
-        <x:v>watch</x:v>
-      </x:c>
-      <x:c r="D20" s="23" t="str">
-        <x:v>https://arxiv.org/abs/2312.00752</x:v>
-      </x:c>
-      <x:c r="E20" s="23" t="str">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="F20" s="23" t="str">
-        <x:v>selective state-space model</x:v>
-      </x:c>
-      <x:c r="G20" s="23" t="str">
-        <x:v>input-dependent state-space selection</x:v>
-      </x:c>
-      <x:c r="H20" s="23" t="str">
-        <x:v>may help only if content-dependent selection is missing</x:v>
-      </x:c>
-      <x:c r="I20" s="23" t="str">
-        <x:v>larger modern implementation can confound capacity</x:v>
-      </x:c>
-      <x:c r="J20" s="23" t="str">
-        <x:v>conditional_after_S4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A21" s="23" t="str">
-        <x:v>NODE-2018</x:v>
-      </x:c>
-      <x:c r="B21" s="23" t="str">
-        <x:v>SC-06</x:v>
-      </x:c>
-      <x:c r="C21" s="23" t="str">
-        <x:v>accepted</x:v>
-      </x:c>
-      <x:c r="D21" s="23" t="str">
-        <x:v>https://proceedings.neurips.cc/paper/2018/hash/69386f6bb1dfed68692a24c8686939b9-Abstract.html</x:v>
-      </x:c>
-      <x:c r="E21" s="23" t="str">
-        <x:v>2018</x:v>
-      </x:c>
-      <x:c r="F21" s="23" t="str">
-        <x:v>Neural ODE</x:v>
-      </x:c>
-      <x:c r="G21" s="23" t="str">
-        <x:v>learned vector field integrated continuously</x:v>
-      </x:c>
-      <x:c r="H21" s="23" t="str">
-        <x:v>matches a physical-state flow prior</x:v>
-      </x:c>
-      <x:c r="I21" s="23" t="str">
-        <x:v>spike inputs are discontinuous controls and solver cost matters</x:v>
-      </x:c>
-      <x:c r="J21" s="23" t="str">
-        <x:v>planned_with_explicit_control_contract</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A22" s="23" t="str">
-        <x:v>NCDE-2020</x:v>
-      </x:c>
-      <x:c r="B22" s="23" t="str">
-        <x:v>SC-06</x:v>
-      </x:c>
-      <x:c r="C22" s="23" t="str">
-        <x:v>watch</x:v>
-      </x:c>
-      <x:c r="D22" s="23" t="str">
-        <x:v>https://proceedings.neurips.cc/paper/2020/hash/4a5876b450b45371f6cfe5047ac8cd45-Abstract.html</x:v>
-      </x:c>
-      <x:c r="E22" s="23" t="str">
-        <x:v>2020</x:v>
-      </x:c>
-      <x:c r="F22" s="23" t="str">
-        <x:v>Neural CDE</x:v>
-      </x:c>
-      <x:c r="G22" s="23" t="str">
-        <x:v>hidden dynamics driven by a control path</x:v>
-      </x:c>
-      <x:c r="H22" s="23" t="str">
-        <x:v>useful if irregular timing or continuous controls enter the task</x:v>
-      </x:c>
-      <x:c r="I22" s="23" t="str">
-        <x:v>current fixed-dt binary event bins weaken its unique advantage</x:v>
-      </x:c>
-      <x:c r="J22" s="23" t="str">
-        <x:v>conditional</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A23" s="23" t="str">
-        <x:v>MPNN-2017</x:v>
-      </x:c>
-      <x:c r="B23" s="23" t="str">
-        <x:v>CB-02;SP-01</x:v>
-      </x:c>
-      <x:c r="C23" s="23" t="str">
-        <x:v>accepted</x:v>
-      </x:c>
-      <x:c r="D23" s="23" t="str">
-        <x:v>https://proceedings.mlr.press/v70/gilmer17a.html</x:v>
-      </x:c>
-      <x:c r="E23" s="23" t="str">
-        <x:v>2017</x:v>
-      </x:c>
-      <x:c r="F23" s="23" t="str">
-        <x:v>message-passing neural network</x:v>
-      </x:c>
-      <x:c r="G23" s="23" t="str">
-        <x:v>shared node updates and edge messages</x:v>
-      </x:c>
-      <x:c r="H23" s="23" t="str">
-        <x:v>matches four-compartment local coupling</x:v>
-      </x:c>
-      <x:c r="I23" s="23" t="str">
-        <x:v>fixed known morphology is tiny and monolithic capacity control is essential</x:v>
-      </x:c>
-      <x:c r="J23" s="23" t="str">
-        <x:v>planned_capability_screen</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A24" s="23" t="str">
-        <x:v>MOE-2017</x:v>
-      </x:c>
-      <x:c r="B24" s="23" t="str">
-        <x:v>HY-01</x:v>
-      </x:c>
-      <x:c r="C24" s="23" t="str">
-        <x:v>watch</x:v>
-      </x:c>
-      <x:c r="D24" s="23" t="str">
-        <x:v>https://arxiv.org/abs/1701.06538</x:v>
-      </x:c>
-      <x:c r="E24" s="23" t="str">
-        <x:v>2017</x:v>
-      </x:c>
-      <x:c r="F24" s="23" t="str">
-        <x:v>sparse mixture of experts</x:v>
-      </x:c>
-      <x:c r="G24" s="23" t="str">
-        <x:v>conditional specialized computation</x:v>
-      </x:c>
-      <x:c r="H24" s="23" t="str">
-        <x:v>may separate rare transition and common regimes</x:v>
-      </x:c>
-      <x:c r="I24" s="23" t="str">
-        <x:v>previous router success did not imply a capable correction expert</x:v>
-      </x:c>
-      <x:c r="J24" s="23" t="str">
-        <x:v>blocked_until_expert_capability</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A25" s="23" t="str">
-        <x:v>CW-RNN-2014</x:v>
-      </x:c>
-      <x:c r="B25" s="23" t="str">
-        <x:v>HY-02</x:v>
-      </x:c>
-      <x:c r="C25" s="23" t="str">
-        <x:v>watch</x:v>
-      </x:c>
-      <x:c r="D25" s="23" t="str">
-        <x:v>https://arxiv.org/abs/1402.3511</x:v>
-      </x:c>
-      <x:c r="E25" s="23" t="str">
-        <x:v>2014</x:v>
-      </x:c>
-      <x:c r="F25" s="23" t="str">
-        <x:v>clockwork recurrent neural network</x:v>
-      </x:c>
-      <x:c r="G25" s="23" t="str">
-        <x:v>modules update at distinct periods</x:v>
-      </x:c>
-      <x:c r="H25" s="23" t="str">
-        <x:v>may reflect measured slow-fast separation</x:v>
-      </x:c>
-      <x:c r="I25" s="23" t="str">
-        <x:v>hard periods may mismatch state-dependent biological timescales</x:v>
-      </x:c>
-      <x:c r="J25" s="23" t="str">
-        <x:v>conditional</x:v>
+        <x:v>SRC-TAXONOMY; SRC-SYSID-LANDSCAPE</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:J1"/>
+    <x:mergeCell ref="A1:G1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>